<commit_message>
feat: actions fetch kookmin 2026-07-25T22:28Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4873" uniqueCount="1409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5065" uniqueCount="1453">
   <si>
     <t>campusCode</t>
   </si>
@@ -4108,10 +4108,142 @@
     <t>소프트웨어융합대학원</t>
   </si>
   <si>
+    <t>7147801</t>
+  </si>
+  <si>
+    <t>자료구조</t>
+  </si>
+  <si>
+    <t>한진섭</t>
+  </si>
+  <si>
     <t>7175701</t>
   </si>
   <si>
     <t>알고리즘특론</t>
+  </si>
+  <si>
+    <t>이지나</t>
+  </si>
+  <si>
+    <t>7241701</t>
+  </si>
+  <si>
+    <t>사용자경험과AI코딩</t>
+  </si>
+  <si>
+    <t>윤종영</t>
+  </si>
+  <si>
+    <t>36296</t>
+  </si>
+  <si>
+    <t>인공지능전공</t>
+  </si>
+  <si>
+    <t>710010a</t>
+  </si>
+  <si>
+    <t>인공지능과비즈니스</t>
+  </si>
+  <si>
+    <t>711610b</t>
+  </si>
+  <si>
+    <t>인공지능자연어처리</t>
+  </si>
+  <si>
+    <t>7142401</t>
+  </si>
+  <si>
+    <t>딥러닝개론</t>
+  </si>
+  <si>
+    <t>7176401</t>
+  </si>
+  <si>
+    <t>인공지능추천시스템</t>
+  </si>
+  <si>
+    <t>36322</t>
+  </si>
+  <si>
+    <t>소프트웨어전공</t>
+  </si>
+  <si>
+    <t>710040b</t>
+  </si>
+  <si>
+    <t>블록체인응용개발</t>
+  </si>
+  <si>
+    <t>7147701</t>
+  </si>
+  <si>
+    <t>소프트웨어공학</t>
+  </si>
+  <si>
+    <t>7175901</t>
+  </si>
+  <si>
+    <t>파이썬매시업프로젝트</t>
+  </si>
+  <si>
+    <t>7176201</t>
+  </si>
+  <si>
+    <t>IoT 기초</t>
+  </si>
+  <si>
+    <t>허대영</t>
+  </si>
+  <si>
+    <t>7264301</t>
+  </si>
+  <si>
+    <t>정보보호개론</t>
+  </si>
+  <si>
+    <t>이수미</t>
+  </si>
+  <si>
+    <t>7264401</t>
+  </si>
+  <si>
+    <t>컴퓨터네트워크의실제</t>
+  </si>
+  <si>
+    <t>36346</t>
+  </si>
+  <si>
+    <t>인공지능응용전공</t>
+  </si>
+  <si>
+    <t>714200b</t>
+  </si>
+  <si>
+    <t>프로그래밍특론</t>
+  </si>
+  <si>
+    <t>714250c</t>
+  </si>
+  <si>
+    <t>데이터분석</t>
+  </si>
+  <si>
+    <t>이정미</t>
+  </si>
+  <si>
+    <t>714270b</t>
+  </si>
+  <si>
+    <t>인공지능수학</t>
+  </si>
+  <si>
+    <t>7264701</t>
+  </si>
+  <si>
+    <t>LLM및프롬프트엔지니어링</t>
   </si>
   <si>
     <t>36379</t>
@@ -4614,7 +4746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M406"/>
+  <dimension ref="A1:M422"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -20838,10 +20970,10 @@
         <v>2</v>
       </c>
       <c r="I396" t="s">
-        <v>166</v>
+        <v>1367</v>
       </c>
       <c r="J396" t="s">
-        <v>166</v>
+        <v>1104</v>
       </c>
       <c r="K396" t="s">
         <v>21</v>
@@ -20855,40 +20987,40 @@
     </row>
     <row r="397" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B397" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C397" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="D397" t="s">
         <v>15</v>
       </c>
       <c r="E397" t="s">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="F397" t="s">
+        <v>1368</v>
+      </c>
+      <c r="G397" t="s">
         <v>1369</v>
       </c>
-      <c r="G397" t="s">
+      <c r="H397">
+        <v>2</v>
+      </c>
+      <c r="I397" t="s">
         <v>1370</v>
       </c>
-      <c r="H397">
-        <v>2</v>
-      </c>
-      <c r="I397" t="s">
-        <v>1371</v>
-      </c>
       <c r="J397" t="s">
-        <v>775</v>
+        <v>767</v>
       </c>
       <c r="K397" t="s">
         <v>21</v>
       </c>
       <c r="L397" t="s">
-        <v>1372</v>
+        <v>166</v>
       </c>
       <c r="M397" t="s">
         <v>23</v>
@@ -20896,40 +21028,40 @@
     </row>
     <row r="398" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B398" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C398" t="s">
+        <v>1363</v>
+      </c>
+      <c r="D398" t="s">
+        <v>15</v>
+      </c>
+      <c r="E398" t="s">
+        <v>36</v>
+      </c>
+      <c r="F398" t="s">
+        <v>1371</v>
+      </c>
+      <c r="G398" t="s">
+        <v>1372</v>
+      </c>
+      <c r="H398">
+        <v>2</v>
+      </c>
+      <c r="I398" t="s">
         <v>1373</v>
       </c>
-      <c r="D398" t="s">
-        <v>1374</v>
-      </c>
-      <c r="E398" t="s">
-        <v>36</v>
-      </c>
-      <c r="F398" t="s">
-        <v>1375</v>
-      </c>
-      <c r="G398" t="s">
-        <v>1376</v>
-      </c>
-      <c r="H398">
-        <v>2</v>
-      </c>
-      <c r="I398" t="s">
-        <v>1377</v>
-      </c>
       <c r="J398" t="s">
-        <v>1378</v>
+        <v>1097</v>
       </c>
       <c r="K398" t="s">
         <v>21</v>
       </c>
       <c r="L398" t="s">
-        <v>1379</v>
+        <v>166</v>
       </c>
       <c r="M398" t="s">
         <v>23</v>
@@ -20937,40 +21069,40 @@
     </row>
     <row r="399" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B399" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C399" t="s">
-        <v>1380</v>
+        <v>1374</v>
       </c>
       <c r="D399" t="s">
-        <v>1381</v>
+        <v>1375</v>
       </c>
       <c r="E399" t="s">
         <v>36</v>
       </c>
       <c r="F399" t="s">
-        <v>1382</v>
+        <v>1376</v>
       </c>
       <c r="G399" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="H399">
         <v>2</v>
       </c>
       <c r="I399" t="s">
-        <v>674</v>
+        <v>166</v>
       </c>
       <c r="J399" t="s">
-        <v>248</v>
+        <v>166</v>
       </c>
       <c r="K399" t="s">
         <v>21</v>
       </c>
       <c r="L399" t="s">
-        <v>1384</v>
+        <v>166</v>
       </c>
       <c r="M399" t="s">
         <v>23</v>
@@ -20978,40 +21110,40 @@
     </row>
     <row r="400" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B400" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C400" t="s">
-        <v>1380</v>
+        <v>1374</v>
       </c>
       <c r="D400" t="s">
-        <v>1381</v>
+        <v>1375</v>
       </c>
       <c r="E400" t="s">
         <v>36</v>
       </c>
       <c r="F400" t="s">
-        <v>1385</v>
+        <v>1378</v>
       </c>
       <c r="G400" t="s">
-        <v>1386</v>
+        <v>1379</v>
       </c>
       <c r="H400">
         <v>2</v>
       </c>
       <c r="I400" t="s">
-        <v>1387</v>
+        <v>166</v>
       </c>
       <c r="J400" t="s">
-        <v>767</v>
+        <v>166</v>
       </c>
       <c r="K400" t="s">
         <v>21</v>
       </c>
       <c r="L400" t="s">
-        <v>1379</v>
+        <v>166</v>
       </c>
       <c r="M400" t="s">
         <v>23</v>
@@ -21019,40 +21151,40 @@
     </row>
     <row r="401" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B401" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C401" t="s">
+        <v>1374</v>
+      </c>
+      <c r="D401" t="s">
+        <v>1375</v>
+      </c>
+      <c r="E401" t="s">
+        <v>36</v>
+      </c>
+      <c r="F401" t="s">
         <v>1380</v>
       </c>
-      <c r="D401" t="s">
+      <c r="G401" t="s">
         <v>1381</v>
       </c>
-      <c r="E401" t="s">
-        <v>36</v>
-      </c>
-      <c r="F401" t="s">
-        <v>1388</v>
-      </c>
-      <c r="G401" t="s">
-        <v>1389</v>
-      </c>
       <c r="H401">
         <v>2</v>
       </c>
       <c r="I401" t="s">
-        <v>1390</v>
+        <v>166</v>
       </c>
       <c r="J401" t="s">
-        <v>1378</v>
+        <v>166</v>
       </c>
       <c r="K401" t="s">
         <v>21</v>
       </c>
       <c r="L401" t="s">
-        <v>1372</v>
+        <v>166</v>
       </c>
       <c r="M401" t="s">
         <v>23</v>
@@ -21060,40 +21192,40 @@
     </row>
     <row r="402" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B402" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C402" t="s">
-        <v>1380</v>
+        <v>1374</v>
       </c>
       <c r="D402" t="s">
-        <v>1381</v>
+        <v>1375</v>
       </c>
       <c r="E402" t="s">
         <v>36</v>
       </c>
       <c r="F402" t="s">
-        <v>1391</v>
+        <v>1382</v>
       </c>
       <c r="G402" t="s">
-        <v>1392</v>
+        <v>1383</v>
       </c>
       <c r="H402">
         <v>2</v>
       </c>
       <c r="I402" t="s">
-        <v>1393</v>
+        <v>166</v>
       </c>
       <c r="J402" t="s">
-        <v>308</v>
+        <v>166</v>
       </c>
       <c r="K402" t="s">
         <v>21</v>
       </c>
       <c r="L402" t="s">
-        <v>1394</v>
+        <v>166</v>
       </c>
       <c r="M402" t="s">
         <v>23</v>
@@ -21101,40 +21233,40 @@
     </row>
     <row r="403" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B403" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C403" t="s">
-        <v>1395</v>
+        <v>1384</v>
       </c>
       <c r="D403" t="s">
-        <v>1396</v>
+        <v>1385</v>
       </c>
       <c r="E403" t="s">
         <v>36</v>
       </c>
       <c r="F403" t="s">
-        <v>1397</v>
+        <v>1386</v>
       </c>
       <c r="G403" t="s">
-        <v>1398</v>
+        <v>1387</v>
       </c>
       <c r="H403">
         <v>2</v>
       </c>
       <c r="I403" t="s">
-        <v>1399</v>
+        <v>166</v>
       </c>
       <c r="J403" t="s">
-        <v>1400</v>
+        <v>166</v>
       </c>
       <c r="K403" t="s">
         <v>21</v>
       </c>
       <c r="L403" t="s">
-        <v>1372</v>
+        <v>166</v>
       </c>
       <c r="M403" t="s">
         <v>23</v>
@@ -21142,40 +21274,40 @@
     </row>
     <row r="404" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B404" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C404" t="s">
-        <v>1395</v>
+        <v>1384</v>
       </c>
       <c r="D404" t="s">
-        <v>1396</v>
+        <v>1385</v>
       </c>
       <c r="E404" t="s">
         <v>36</v>
       </c>
       <c r="F404" t="s">
-        <v>1401</v>
+        <v>1388</v>
       </c>
       <c r="G404" t="s">
-        <v>1402</v>
+        <v>1389</v>
       </c>
       <c r="H404">
         <v>2</v>
       </c>
       <c r="I404" t="s">
-        <v>1399</v>
+        <v>1370</v>
       </c>
       <c r="J404" t="s">
-        <v>248</v>
+        <v>166</v>
       </c>
       <c r="K404" t="s">
         <v>21</v>
       </c>
       <c r="L404" t="s">
-        <v>1394</v>
+        <v>166</v>
       </c>
       <c r="M404" t="s">
         <v>23</v>
@@ -21183,40 +21315,40 @@
     </row>
     <row r="405" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B405" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C405" t="s">
-        <v>1395</v>
+        <v>1384</v>
       </c>
       <c r="D405" t="s">
-        <v>1396</v>
+        <v>1385</v>
       </c>
       <c r="E405" t="s">
         <v>36</v>
       </c>
       <c r="F405" t="s">
-        <v>1403</v>
+        <v>1390</v>
       </c>
       <c r="G405" t="s">
-        <v>1404</v>
+        <v>1391</v>
       </c>
       <c r="H405">
         <v>2</v>
       </c>
       <c r="I405" t="s">
-        <v>1371</v>
+        <v>166</v>
       </c>
       <c r="J405" t="s">
-        <v>1405</v>
+        <v>166</v>
       </c>
       <c r="K405" t="s">
         <v>21</v>
       </c>
       <c r="L405" t="s">
-        <v>1379</v>
+        <v>166</v>
       </c>
       <c r="M405" t="s">
         <v>23</v>
@@ -21224,42 +21356,698 @@
     </row>
     <row r="406" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="B406" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C406" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D406" t="s">
+        <v>1385</v>
+      </c>
+      <c r="E406" t="s">
+        <v>36</v>
+      </c>
+      <c r="F406" t="s">
+        <v>1392</v>
+      </c>
+      <c r="G406" t="s">
+        <v>1393</v>
+      </c>
+      <c r="H406">
+        <v>2</v>
+      </c>
+      <c r="I406" t="s">
+        <v>1394</v>
+      </c>
+      <c r="J406" t="s">
+        <v>166</v>
+      </c>
+      <c r="K406" t="s">
+        <v>21</v>
+      </c>
+      <c r="L406" t="s">
+        <v>166</v>
+      </c>
+      <c r="M406" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="407" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B407" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C407" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D407" t="s">
+        <v>1385</v>
+      </c>
+      <c r="E407" t="s">
+        <v>36</v>
+      </c>
+      <c r="F407" t="s">
         <v>1395</v>
       </c>
-      <c r="D406" t="s">
+      <c r="G407" t="s">
         <v>1396</v>
       </c>
-      <c r="E406" t="s">
-        <v>36</v>
-      </c>
-      <c r="F406" t="s">
+      <c r="H407">
+        <v>2</v>
+      </c>
+      <c r="I407" t="s">
+        <v>1397</v>
+      </c>
+      <c r="J407" t="s">
+        <v>166</v>
+      </c>
+      <c r="K407" t="s">
+        <v>21</v>
+      </c>
+      <c r="L407" t="s">
+        <v>166</v>
+      </c>
+      <c r="M407" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="408" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B408" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C408" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D408" t="s">
+        <v>1385</v>
+      </c>
+      <c r="E408" t="s">
+        <v>36</v>
+      </c>
+      <c r="F408" t="s">
+        <v>1398</v>
+      </c>
+      <c r="G408" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H408">
+        <v>2</v>
+      </c>
+      <c r="I408" t="s">
+        <v>166</v>
+      </c>
+      <c r="J408" t="s">
+        <v>166</v>
+      </c>
+      <c r="K408" t="s">
+        <v>21</v>
+      </c>
+      <c r="L408" t="s">
+        <v>166</v>
+      </c>
+      <c r="M408" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="409" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B409" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C409" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D409" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E409" t="s">
+        <v>36</v>
+      </c>
+      <c r="F409" t="s">
+        <v>1402</v>
+      </c>
+      <c r="G409" t="s">
+        <v>1403</v>
+      </c>
+      <c r="H409">
+        <v>2</v>
+      </c>
+      <c r="I409" t="s">
+        <v>166</v>
+      </c>
+      <c r="J409" t="s">
+        <v>166</v>
+      </c>
+      <c r="K409" t="s">
+        <v>21</v>
+      </c>
+      <c r="L409" t="s">
+        <v>166</v>
+      </c>
+      <c r="M409" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="410" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B410" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C410" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D410" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E410" t="s">
+        <v>36</v>
+      </c>
+      <c r="F410" t="s">
+        <v>1404</v>
+      </c>
+      <c r="G410" t="s">
+        <v>1405</v>
+      </c>
+      <c r="H410">
+        <v>2</v>
+      </c>
+      <c r="I410" t="s">
         <v>1406</v>
       </c>
-      <c r="G406" t="s">
+      <c r="J410" t="s">
+        <v>166</v>
+      </c>
+      <c r="K410" t="s">
+        <v>21</v>
+      </c>
+      <c r="L410" t="s">
+        <v>166</v>
+      </c>
+      <c r="M410" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="411" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B411" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C411" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D411" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E411" t="s">
+        <v>36</v>
+      </c>
+      <c r="F411" t="s">
         <v>1407</v>
       </c>
-      <c r="H406">
-        <v>2</v>
-      </c>
-      <c r="I406" t="s">
+      <c r="G411" t="s">
         <v>1408</v>
       </c>
-      <c r="J406" t="s">
+      <c r="H411">
+        <v>2</v>
+      </c>
+      <c r="I411" t="s">
+        <v>166</v>
+      </c>
+      <c r="J411" t="s">
+        <v>166</v>
+      </c>
+      <c r="K411" t="s">
+        <v>21</v>
+      </c>
+      <c r="L411" t="s">
+        <v>166</v>
+      </c>
+      <c r="M411" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="412" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B412" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C412" t="s">
+        <v>1400</v>
+      </c>
+      <c r="D412" t="s">
+        <v>1401</v>
+      </c>
+      <c r="E412" t="s">
+        <v>36</v>
+      </c>
+      <c r="F412" t="s">
+        <v>1409</v>
+      </c>
+      <c r="G412" t="s">
+        <v>1410</v>
+      </c>
+      <c r="H412">
+        <v>2</v>
+      </c>
+      <c r="I412" t="s">
+        <v>166</v>
+      </c>
+      <c r="J412" t="s">
+        <v>166</v>
+      </c>
+      <c r="K412" t="s">
+        <v>21</v>
+      </c>
+      <c r="L412" t="s">
+        <v>166</v>
+      </c>
+      <c r="M412" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="413" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B413" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C413" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D413" t="s">
+        <v>15</v>
+      </c>
+      <c r="E413" t="s">
+        <v>95</v>
+      </c>
+      <c r="F413" t="s">
+        <v>1413</v>
+      </c>
+      <c r="G413" t="s">
+        <v>1414</v>
+      </c>
+      <c r="H413">
+        <v>2</v>
+      </c>
+      <c r="I413" t="s">
+        <v>1415</v>
+      </c>
+      <c r="J413" t="s">
+        <v>775</v>
+      </c>
+      <c r="K413" t="s">
+        <v>21</v>
+      </c>
+      <c r="L413" t="s">
+        <v>1416</v>
+      </c>
+      <c r="M413" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="414" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B414" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C414" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D414" t="s">
+        <v>1418</v>
+      </c>
+      <c r="E414" t="s">
+        <v>36</v>
+      </c>
+      <c r="F414" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G414" t="s">
+        <v>1420</v>
+      </c>
+      <c r="H414">
+        <v>2</v>
+      </c>
+      <c r="I414" t="s">
+        <v>1421</v>
+      </c>
+      <c r="J414" t="s">
+        <v>1422</v>
+      </c>
+      <c r="K414" t="s">
+        <v>21</v>
+      </c>
+      <c r="L414" t="s">
+        <v>1423</v>
+      </c>
+      <c r="M414" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="415" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B415" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C415" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D415" t="s">
+        <v>1425</v>
+      </c>
+      <c r="E415" t="s">
+        <v>36</v>
+      </c>
+      <c r="F415" t="s">
+        <v>1426</v>
+      </c>
+      <c r="G415" t="s">
+        <v>1427</v>
+      </c>
+      <c r="H415">
+        <v>2</v>
+      </c>
+      <c r="I415" t="s">
+        <v>674</v>
+      </c>
+      <c r="J415" t="s">
+        <v>248</v>
+      </c>
+      <c r="K415" t="s">
+        <v>21</v>
+      </c>
+      <c r="L415" t="s">
+        <v>1428</v>
+      </c>
+      <c r="M415" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="416" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C416" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D416" t="s">
+        <v>1425</v>
+      </c>
+      <c r="E416" t="s">
+        <v>36</v>
+      </c>
+      <c r="F416" t="s">
+        <v>1429</v>
+      </c>
+      <c r="G416" t="s">
+        <v>1430</v>
+      </c>
+      <c r="H416">
+        <v>2</v>
+      </c>
+      <c r="I416" t="s">
+        <v>1431</v>
+      </c>
+      <c r="J416" t="s">
         <v>767</v>
       </c>
-      <c r="K406" t="s">
-        <v>21</v>
-      </c>
-      <c r="L406" t="s">
-        <v>1372</v>
-      </c>
-      <c r="M406" t="s">
+      <c r="K416" t="s">
+        <v>21</v>
+      </c>
+      <c r="L416" t="s">
+        <v>1423</v>
+      </c>
+      <c r="M416" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="417" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B417" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C417" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D417" t="s">
+        <v>1425</v>
+      </c>
+      <c r="E417" t="s">
+        <v>36</v>
+      </c>
+      <c r="F417" t="s">
+        <v>1432</v>
+      </c>
+      <c r="G417" t="s">
+        <v>1433</v>
+      </c>
+      <c r="H417">
+        <v>2</v>
+      </c>
+      <c r="I417" t="s">
+        <v>1434</v>
+      </c>
+      <c r="J417" t="s">
+        <v>1422</v>
+      </c>
+      <c r="K417" t="s">
+        <v>21</v>
+      </c>
+      <c r="L417" t="s">
+        <v>1416</v>
+      </c>
+      <c r="M417" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="418" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B418" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C418" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D418" t="s">
+        <v>1425</v>
+      </c>
+      <c r="E418" t="s">
+        <v>36</v>
+      </c>
+      <c r="F418" t="s">
+        <v>1435</v>
+      </c>
+      <c r="G418" t="s">
+        <v>1436</v>
+      </c>
+      <c r="H418">
+        <v>2</v>
+      </c>
+      <c r="I418" t="s">
+        <v>1437</v>
+      </c>
+      <c r="J418" t="s">
+        <v>308</v>
+      </c>
+      <c r="K418" t="s">
+        <v>21</v>
+      </c>
+      <c r="L418" t="s">
+        <v>1438</v>
+      </c>
+      <c r="M418" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="419" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B419" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C419" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D419" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E419" t="s">
+        <v>36</v>
+      </c>
+      <c r="F419" t="s">
+        <v>1441</v>
+      </c>
+      <c r="G419" t="s">
+        <v>1442</v>
+      </c>
+      <c r="H419">
+        <v>2</v>
+      </c>
+      <c r="I419" t="s">
+        <v>1443</v>
+      </c>
+      <c r="J419" t="s">
+        <v>1444</v>
+      </c>
+      <c r="K419" t="s">
+        <v>21</v>
+      </c>
+      <c r="L419" t="s">
+        <v>1416</v>
+      </c>
+      <c r="M419" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="420" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B420" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C420" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D420" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E420" t="s">
+        <v>36</v>
+      </c>
+      <c r="F420" t="s">
+        <v>1445</v>
+      </c>
+      <c r="G420" t="s">
+        <v>1446</v>
+      </c>
+      <c r="H420">
+        <v>2</v>
+      </c>
+      <c r="I420" t="s">
+        <v>1443</v>
+      </c>
+      <c r="J420" t="s">
+        <v>248</v>
+      </c>
+      <c r="K420" t="s">
+        <v>21</v>
+      </c>
+      <c r="L420" t="s">
+        <v>1438</v>
+      </c>
+      <c r="M420" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="421" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B421" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C421" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D421" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E421" t="s">
+        <v>36</v>
+      </c>
+      <c r="F421" t="s">
+        <v>1447</v>
+      </c>
+      <c r="G421" t="s">
+        <v>1448</v>
+      </c>
+      <c r="H421">
+        <v>2</v>
+      </c>
+      <c r="I421" t="s">
+        <v>1415</v>
+      </c>
+      <c r="J421" t="s">
+        <v>1449</v>
+      </c>
+      <c r="K421" t="s">
+        <v>21</v>
+      </c>
+      <c r="L421" t="s">
+        <v>1423</v>
+      </c>
+      <c r="M421" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="422" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B422" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C422" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D422" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E422" t="s">
+        <v>36</v>
+      </c>
+      <c r="F422" t="s">
+        <v>1450</v>
+      </c>
+      <c r="G422" t="s">
+        <v>1451</v>
+      </c>
+      <c r="H422">
+        <v>2</v>
+      </c>
+      <c r="I422" t="s">
+        <v>1452</v>
+      </c>
+      <c r="J422" t="s">
+        <v>767</v>
+      </c>
+      <c r="K422" t="s">
+        <v>21</v>
+      </c>
+      <c r="L422" t="s">
+        <v>1416</v>
+      </c>
+      <c r="M422" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-08-08T21:57Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12085" uniqueCount="2957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12085" uniqueCount="2961">
   <si>
     <t>campusCode</t>
   </si>
@@ -8545,6 +8545,9 @@
     <t>한진섭</t>
   </si>
   <si>
+    <t>미래관4층47호실</t>
+  </si>
+  <si>
     <t>7175701</t>
   </si>
   <si>
@@ -8560,12 +8563,18 @@
     <t>논문/프로젝트I</t>
   </si>
   <si>
+    <t>미래관4층45호실</t>
+  </si>
+  <si>
     <t>7223501</t>
   </si>
   <si>
     <t>논문/프로젝트II</t>
   </si>
   <si>
+    <t>미래관4층24호실</t>
+  </si>
+  <si>
     <t>김준호</t>
   </si>
   <si>
@@ -8729,6 +8738,9 @@
   </si>
   <si>
     <t>이창우</t>
+  </si>
+  <si>
+    <t>미래관6층11호실</t>
   </si>
   <si>
     <t>7208601</t>
@@ -48943,7 +48955,7 @@
         <v>21</v>
       </c>
       <c r="L968" t="s">
-        <v>116</v>
+        <v>2844</v>
       </c>
       <c r="M968" t="s">
         <v>23</v>
@@ -48966,16 +48978,16 @@
         <v>16</v>
       </c>
       <c r="F969" t="s">
-        <v>2844</v>
+        <v>2845</v>
       </c>
       <c r="G969" t="s">
-        <v>2845</v>
+        <v>2846</v>
       </c>
       <c r="H969">
         <v>2</v>
       </c>
       <c r="I969" t="s">
-        <v>2846</v>
+        <v>2847</v>
       </c>
       <c r="J969" t="s">
         <v>2209</v>
@@ -48984,7 +48996,7 @@
         <v>21</v>
       </c>
       <c r="L969" t="s">
-        <v>116</v>
+        <v>2844</v>
       </c>
       <c r="M969" t="s">
         <v>23</v>
@@ -49007,10 +49019,10 @@
         <v>16</v>
       </c>
       <c r="F970" t="s">
-        <v>2847</v>
+        <v>2848</v>
       </c>
       <c r="G970" t="s">
-        <v>2848</v>
+        <v>2849</v>
       </c>
       <c r="H970">
         <v>2</v>
@@ -49025,7 +49037,7 @@
         <v>21</v>
       </c>
       <c r="L970" t="s">
-        <v>116</v>
+        <v>2850</v>
       </c>
       <c r="M970" t="s">
         <v>23</v>
@@ -49048,10 +49060,10 @@
         <v>16</v>
       </c>
       <c r="F971" t="s">
-        <v>2849</v>
+        <v>2851</v>
       </c>
       <c r="G971" t="s">
-        <v>2850</v>
+        <v>2852</v>
       </c>
       <c r="H971">
         <v>2</v>
@@ -49066,7 +49078,7 @@
         <v>21</v>
       </c>
       <c r="L971" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M971" t="s">
         <v>23</v>
@@ -49089,10 +49101,10 @@
         <v>16</v>
       </c>
       <c r="F972" t="s">
-        <v>2849</v>
+        <v>2851</v>
       </c>
       <c r="G972" t="s">
-        <v>2850</v>
+        <v>2852</v>
       </c>
       <c r="H972">
         <v>2</v>
@@ -49107,7 +49119,7 @@
         <v>21</v>
       </c>
       <c r="L972" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M972" t="s">
         <v>623</v>
@@ -49130,16 +49142,16 @@
         <v>16</v>
       </c>
       <c r="F973" t="s">
-        <v>2849</v>
+        <v>2851</v>
       </c>
       <c r="G973" t="s">
-        <v>2850</v>
+        <v>2852</v>
       </c>
       <c r="H973">
         <v>2</v>
       </c>
       <c r="I973" t="s">
-        <v>2851</v>
+        <v>2854</v>
       </c>
       <c r="J973" t="s">
         <v>2218</v>
@@ -49148,7 +49160,7 @@
         <v>21</v>
       </c>
       <c r="L973" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M973" t="s">
         <v>624</v>
@@ -49171,16 +49183,16 @@
         <v>16</v>
       </c>
       <c r="F974" t="s">
-        <v>2849</v>
+        <v>2851</v>
       </c>
       <c r="G974" t="s">
-        <v>2850</v>
+        <v>2852</v>
       </c>
       <c r="H974">
         <v>2</v>
       </c>
       <c r="I974" t="s">
-        <v>2852</v>
+        <v>2855</v>
       </c>
       <c r="J974" t="s">
         <v>2209</v>
@@ -49189,7 +49201,7 @@
         <v>21</v>
       </c>
       <c r="L974" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M974" t="s">
         <v>625</v>
@@ -49212,16 +49224,16 @@
         <v>16</v>
       </c>
       <c r="F975" t="s">
-        <v>2849</v>
+        <v>2851</v>
       </c>
       <c r="G975" t="s">
-        <v>2850</v>
+        <v>2852</v>
       </c>
       <c r="H975">
         <v>2</v>
       </c>
       <c r="I975" t="s">
-        <v>2853</v>
+        <v>2856</v>
       </c>
       <c r="J975" t="s">
         <v>2213</v>
@@ -49230,7 +49242,7 @@
         <v>21</v>
       </c>
       <c r="L975" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M975" t="s">
         <v>626</v>
@@ -49253,16 +49265,16 @@
         <v>16</v>
       </c>
       <c r="F976" t="s">
-        <v>2854</v>
+        <v>2857</v>
       </c>
       <c r="G976" t="s">
-        <v>2855</v>
+        <v>2858</v>
       </c>
       <c r="H976">
         <v>2</v>
       </c>
       <c r="I976" t="s">
-        <v>2852</v>
+        <v>2855</v>
       </c>
       <c r="J976" t="s">
         <v>2363</v>
@@ -49271,7 +49283,7 @@
         <v>21</v>
       </c>
       <c r="L976" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M976" t="s">
         <v>23</v>
@@ -49294,25 +49306,25 @@
         <v>16</v>
       </c>
       <c r="F977" t="s">
-        <v>2856</v>
+        <v>2859</v>
       </c>
       <c r="G977" t="s">
-        <v>2857</v>
+        <v>2860</v>
       </c>
       <c r="H977">
         <v>2</v>
       </c>
       <c r="I977" t="s">
-        <v>2858</v>
+        <v>2861</v>
       </c>
       <c r="J977" t="s">
-        <v>2859</v>
+        <v>2862</v>
       </c>
       <c r="K977" t="s">
         <v>21</v>
       </c>
       <c r="L977" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M977" t="s">
         <v>23</v>
@@ -49326,25 +49338,25 @@
         <v>2840</v>
       </c>
       <c r="C978" t="s">
-        <v>2860</v>
+        <v>2863</v>
       </c>
       <c r="D978" t="s">
-        <v>2861</v>
+        <v>2864</v>
       </c>
       <c r="E978" t="s">
         <v>16</v>
       </c>
       <c r="F978" t="s">
-        <v>2862</v>
+        <v>2865</v>
       </c>
       <c r="G978" t="s">
-        <v>2863</v>
+        <v>2866</v>
       </c>
       <c r="H978">
         <v>2</v>
       </c>
       <c r="I978" t="s">
-        <v>2852</v>
+        <v>2855</v>
       </c>
       <c r="J978" t="s">
         <v>2387</v>
@@ -49353,7 +49365,7 @@
         <v>21</v>
       </c>
       <c r="L978" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M978" t="s">
         <v>23</v>
@@ -49367,25 +49379,25 @@
         <v>2840</v>
       </c>
       <c r="C979" t="s">
-        <v>2860</v>
+        <v>2863</v>
       </c>
       <c r="D979" t="s">
-        <v>2861</v>
+        <v>2864</v>
       </c>
       <c r="E979" t="s">
         <v>16</v>
       </c>
       <c r="F979" t="s">
-        <v>2864</v>
+        <v>2867</v>
       </c>
       <c r="G979" t="s">
-        <v>2865</v>
+        <v>2868</v>
       </c>
       <c r="H979">
         <v>2</v>
       </c>
       <c r="I979" t="s">
-        <v>2866</v>
+        <v>2869</v>
       </c>
       <c r="J979" t="s">
         <v>2218</v>
@@ -49394,7 +49406,7 @@
         <v>21</v>
       </c>
       <c r="L979" t="s">
-        <v>116</v>
+        <v>2549</v>
       </c>
       <c r="M979" t="s">
         <v>23</v>
@@ -49408,25 +49420,25 @@
         <v>2840</v>
       </c>
       <c r="C980" t="s">
-        <v>2860</v>
+        <v>2863</v>
       </c>
       <c r="D980" t="s">
-        <v>2861</v>
+        <v>2864</v>
       </c>
       <c r="E980" t="s">
         <v>16</v>
       </c>
       <c r="F980" t="s">
-        <v>2867</v>
+        <v>2870</v>
       </c>
       <c r="G980" t="s">
-        <v>2868</v>
+        <v>2871</v>
       </c>
       <c r="H980">
         <v>2</v>
       </c>
       <c r="I980" t="s">
-        <v>2869</v>
+        <v>2872</v>
       </c>
       <c r="J980" t="s">
         <v>2363</v>
@@ -49435,7 +49447,7 @@
         <v>21</v>
       </c>
       <c r="L980" t="s">
-        <v>116</v>
+        <v>2844</v>
       </c>
       <c r="M980" t="s">
         <v>23</v>
@@ -49449,25 +49461,25 @@
         <v>2840</v>
       </c>
       <c r="C981" t="s">
-        <v>2860</v>
+        <v>2863</v>
       </c>
       <c r="D981" t="s">
-        <v>2861</v>
+        <v>2864</v>
       </c>
       <c r="E981" t="s">
         <v>16</v>
       </c>
       <c r="F981" t="s">
-        <v>2870</v>
+        <v>2873</v>
       </c>
       <c r="G981" t="s">
-        <v>2871</v>
+        <v>2874</v>
       </c>
       <c r="H981">
         <v>2</v>
       </c>
       <c r="I981" t="s">
-        <v>2872</v>
+        <v>2875</v>
       </c>
       <c r="J981" t="s">
         <v>2387</v>
@@ -49476,7 +49488,7 @@
         <v>21</v>
       </c>
       <c r="L981" t="s">
-        <v>116</v>
+        <v>2549</v>
       </c>
       <c r="M981" t="s">
         <v>23</v>
@@ -49490,25 +49502,25 @@
         <v>2840</v>
       </c>
       <c r="C982" t="s">
-        <v>2860</v>
+        <v>2863</v>
       </c>
       <c r="D982" t="s">
-        <v>2861</v>
+        <v>2864</v>
       </c>
       <c r="E982" t="s">
         <v>16</v>
       </c>
       <c r="F982" t="s">
-        <v>2873</v>
+        <v>2876</v>
       </c>
       <c r="G982" t="s">
-        <v>2874</v>
+        <v>2877</v>
       </c>
       <c r="H982">
         <v>2</v>
       </c>
       <c r="I982" t="s">
-        <v>2875</v>
+        <v>2878</v>
       </c>
       <c r="J982" t="s">
         <v>2218</v>
@@ -49517,7 +49529,7 @@
         <v>21</v>
       </c>
       <c r="L982" t="s">
-        <v>116</v>
+        <v>2468</v>
       </c>
       <c r="M982" t="s">
         <v>23</v>
@@ -49531,25 +49543,25 @@
         <v>2840</v>
       </c>
       <c r="C983" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D983" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E983" t="s">
         <v>16</v>
       </c>
       <c r="F983" t="s">
-        <v>2878</v>
+        <v>2881</v>
       </c>
       <c r="G983" t="s">
-        <v>2879</v>
+        <v>2882</v>
       </c>
       <c r="H983">
         <v>2</v>
       </c>
       <c r="I983" t="s">
-        <v>2880</v>
+        <v>2883</v>
       </c>
       <c r="J983" t="s">
         <v>2387</v>
@@ -49558,7 +49570,7 @@
         <v>21</v>
       </c>
       <c r="L983" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M983" t="s">
         <v>23</v>
@@ -49572,25 +49584,25 @@
         <v>2840</v>
       </c>
       <c r="C984" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D984" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E984" t="s">
         <v>16</v>
       </c>
       <c r="F984" t="s">
-        <v>2881</v>
+        <v>2884</v>
       </c>
       <c r="G984" t="s">
-        <v>2882</v>
+        <v>2885</v>
       </c>
       <c r="H984">
         <v>2</v>
       </c>
       <c r="I984" t="s">
-        <v>2846</v>
+        <v>2847</v>
       </c>
       <c r="J984" t="s">
         <v>2218</v>
@@ -49599,7 +49611,7 @@
         <v>21</v>
       </c>
       <c r="L984" t="s">
-        <v>116</v>
+        <v>2844</v>
       </c>
       <c r="M984" t="s">
         <v>23</v>
@@ -49613,25 +49625,25 @@
         <v>2840</v>
       </c>
       <c r="C985" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D985" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E985" t="s">
         <v>16</v>
       </c>
       <c r="F985" t="s">
-        <v>2883</v>
+        <v>2886</v>
       </c>
       <c r="G985" t="s">
-        <v>2884</v>
+        <v>2887</v>
       </c>
       <c r="H985">
         <v>2</v>
       </c>
       <c r="I985" t="s">
-        <v>2885</v>
+        <v>2888</v>
       </c>
       <c r="J985" t="s">
         <v>2387</v>
@@ -49640,7 +49652,7 @@
         <v>21</v>
       </c>
       <c r="L985" t="s">
-        <v>116</v>
+        <v>2468</v>
       </c>
       <c r="M985" t="s">
         <v>23</v>
@@ -49654,19 +49666,19 @@
         <v>2840</v>
       </c>
       <c r="C986" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D986" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E986" t="s">
         <v>16</v>
       </c>
       <c r="F986" t="s">
-        <v>2886</v>
+        <v>2889</v>
       </c>
       <c r="G986" t="s">
-        <v>2887</v>
+        <v>2890</v>
       </c>
       <c r="H986">
         <v>2</v>
@@ -49681,7 +49693,7 @@
         <v>21</v>
       </c>
       <c r="L986" t="s">
-        <v>116</v>
+        <v>2850</v>
       </c>
       <c r="M986" t="s">
         <v>23</v>
@@ -49695,16 +49707,16 @@
         <v>2840</v>
       </c>
       <c r="C987" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D987" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E987" t="s">
         <v>16</v>
       </c>
       <c r="F987" t="s">
-        <v>2888</v>
+        <v>2891</v>
       </c>
       <c r="G987" t="s">
         <v>452</v>
@@ -49713,7 +49725,7 @@
         <v>2</v>
       </c>
       <c r="I987" t="s">
-        <v>2889</v>
+        <v>2892</v>
       </c>
       <c r="J987" t="s">
         <v>2209</v>
@@ -49722,7 +49734,7 @@
         <v>21</v>
       </c>
       <c r="L987" t="s">
-        <v>116</v>
+        <v>2549</v>
       </c>
       <c r="M987" t="s">
         <v>23</v>
@@ -49736,25 +49748,25 @@
         <v>2840</v>
       </c>
       <c r="C988" t="s">
-        <v>2876</v>
+        <v>2879</v>
       </c>
       <c r="D988" t="s">
-        <v>2877</v>
+        <v>2880</v>
       </c>
       <c r="E988" t="s">
         <v>16</v>
       </c>
       <c r="F988" t="s">
-        <v>2890</v>
+        <v>2893</v>
       </c>
       <c r="G988" t="s">
-        <v>2891</v>
+        <v>2894</v>
       </c>
       <c r="H988">
         <v>2</v>
       </c>
       <c r="I988" t="s">
-        <v>2852</v>
+        <v>2855</v>
       </c>
       <c r="J988" t="s">
         <v>2218</v>
@@ -49763,7 +49775,7 @@
         <v>21</v>
       </c>
       <c r="L988" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M988" t="s">
         <v>23</v>
@@ -49777,34 +49789,34 @@
         <v>2840</v>
       </c>
       <c r="C989" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D989" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E989" t="s">
         <v>16</v>
       </c>
       <c r="F989" t="s">
-        <v>2894</v>
+        <v>2897</v>
       </c>
       <c r="G989" t="s">
-        <v>2895</v>
+        <v>2898</v>
       </c>
       <c r="H989">
         <v>2</v>
       </c>
       <c r="I989" t="s">
-        <v>2885</v>
+        <v>2888</v>
       </c>
       <c r="J989" t="s">
-        <v>2896</v>
+        <v>2899</v>
       </c>
       <c r="K989" t="s">
         <v>21</v>
       </c>
       <c r="L989" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M989" t="s">
         <v>23</v>
@@ -49818,34 +49830,34 @@
         <v>2840</v>
       </c>
       <c r="C990" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D990" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E990" t="s">
         <v>16</v>
       </c>
       <c r="F990" t="s">
-        <v>2897</v>
+        <v>2900</v>
       </c>
       <c r="G990" t="s">
-        <v>2898</v>
+        <v>2901</v>
       </c>
       <c r="H990">
         <v>2</v>
       </c>
       <c r="I990" t="s">
-        <v>2899</v>
+        <v>2902</v>
       </c>
       <c r="J990" t="s">
-        <v>2900</v>
+        <v>2903</v>
       </c>
       <c r="K990" t="s">
         <v>21</v>
       </c>
       <c r="L990" t="s">
-        <v>116</v>
+        <v>2853</v>
       </c>
       <c r="M990" t="s">
         <v>23</v>
@@ -49859,25 +49871,25 @@
         <v>2840</v>
       </c>
       <c r="C991" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D991" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E991" t="s">
         <v>16</v>
       </c>
       <c r="F991" t="s">
-        <v>2901</v>
+        <v>2904</v>
       </c>
       <c r="G991" t="s">
-        <v>2902</v>
+        <v>2905</v>
       </c>
       <c r="H991">
         <v>2</v>
       </c>
       <c r="I991" t="s">
-        <v>2880</v>
+        <v>2883</v>
       </c>
       <c r="J991" t="s">
         <v>2213</v>
@@ -49886,7 +49898,7 @@
         <v>21</v>
       </c>
       <c r="L991" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M991" t="s">
         <v>23</v>
@@ -49900,25 +49912,25 @@
         <v>2840</v>
       </c>
       <c r="C992" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D992" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E992" t="s">
         <v>16</v>
       </c>
       <c r="F992" t="s">
-        <v>2903</v>
+        <v>2906</v>
       </c>
       <c r="G992" t="s">
-        <v>2904</v>
+        <v>2907</v>
       </c>
       <c r="H992">
         <v>2</v>
       </c>
       <c r="I992" t="s">
-        <v>2905</v>
+        <v>2908</v>
       </c>
       <c r="J992" t="s">
         <v>2363</v>
@@ -49927,7 +49939,7 @@
         <v>21</v>
       </c>
       <c r="L992" t="s">
-        <v>116</v>
+        <v>2909</v>
       </c>
       <c r="M992" t="s">
         <v>23</v>
@@ -49941,25 +49953,25 @@
         <v>2840</v>
       </c>
       <c r="C993" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D993" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E993" t="s">
         <v>16</v>
       </c>
       <c r="F993" t="s">
-        <v>2906</v>
+        <v>2910</v>
       </c>
       <c r="G993" t="s">
-        <v>2907</v>
+        <v>2911</v>
       </c>
       <c r="H993">
         <v>2</v>
       </c>
       <c r="I993" t="s">
-        <v>2899</v>
+        <v>2902</v>
       </c>
       <c r="J993" t="s">
         <v>2218</v>
@@ -49968,7 +49980,7 @@
         <v>21</v>
       </c>
       <c r="L993" t="s">
-        <v>116</v>
+        <v>2909</v>
       </c>
       <c r="M993" t="s">
         <v>23</v>
@@ -49982,25 +49994,25 @@
         <v>2840</v>
       </c>
       <c r="C994" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D994" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E994" t="s">
         <v>16</v>
       </c>
       <c r="F994" t="s">
-        <v>2908</v>
+        <v>2912</v>
       </c>
       <c r="G994" t="s">
-        <v>2909</v>
+        <v>2913</v>
       </c>
       <c r="H994">
         <v>2</v>
       </c>
       <c r="I994" t="s">
-        <v>2853</v>
+        <v>2856</v>
       </c>
       <c r="J994" t="s">
         <v>2363</v>
@@ -50009,7 +50021,7 @@
         <v>21</v>
       </c>
       <c r="L994" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M994" t="s">
         <v>23</v>
@@ -50023,25 +50035,25 @@
         <v>2840</v>
       </c>
       <c r="C995" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D995" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E995" t="s">
         <v>16</v>
       </c>
       <c r="F995" t="s">
-        <v>2910</v>
+        <v>2914</v>
       </c>
       <c r="G995" t="s">
-        <v>2911</v>
+        <v>2915</v>
       </c>
       <c r="H995">
         <v>2</v>
       </c>
       <c r="I995" t="s">
-        <v>2912</v>
+        <v>2916</v>
       </c>
       <c r="J995" t="s">
         <v>2209</v>
@@ -50050,7 +50062,7 @@
         <v>21</v>
       </c>
       <c r="L995" t="s">
-        <v>116</v>
+        <v>2909</v>
       </c>
       <c r="M995" t="s">
         <v>23</v>
@@ -50064,25 +50076,25 @@
         <v>2840</v>
       </c>
       <c r="C996" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D996" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E996" t="s">
         <v>16</v>
       </c>
       <c r="F996" t="s">
-        <v>2913</v>
+        <v>2917</v>
       </c>
       <c r="G996" t="s">
-        <v>2914</v>
+        <v>2918</v>
       </c>
       <c r="H996">
         <v>2</v>
       </c>
       <c r="I996" t="s">
-        <v>2866</v>
+        <v>2869</v>
       </c>
       <c r="J996" t="s">
         <v>2209</v>
@@ -50091,7 +50103,7 @@
         <v>21</v>
       </c>
       <c r="L996" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="M996" t="s">
         <v>23</v>
@@ -50105,25 +50117,25 @@
         <v>2840</v>
       </c>
       <c r="C997" t="s">
-        <v>2892</v>
+        <v>2895</v>
       </c>
       <c r="D997" t="s">
-        <v>2893</v>
+        <v>2896</v>
       </c>
       <c r="E997" t="s">
         <v>16</v>
       </c>
       <c r="F997" t="s">
-        <v>2915</v>
+        <v>2919</v>
       </c>
       <c r="G997" t="s">
-        <v>2916</v>
+        <v>2920</v>
       </c>
       <c r="H997">
         <v>2</v>
       </c>
       <c r="I997" t="s">
-        <v>2853</v>
+        <v>2856</v>
       </c>
       <c r="J997" t="s">
         <v>2387</v>
@@ -50132,7 +50144,7 @@
         <v>21</v>
       </c>
       <c r="L997" t="s">
-        <v>116</v>
+        <v>2909</v>
       </c>
       <c r="M997" t="s">
         <v>23</v>
@@ -50140,13 +50152,13 @@
     </row>
     <row r="998" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A998" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B998" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C998" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="D998" t="s">
         <v>15</v>
@@ -50155,16 +50167,16 @@
         <v>1583</v>
       </c>
       <c r="F998" t="s">
-        <v>2919</v>
+        <v>2923</v>
       </c>
       <c r="G998" t="s">
-        <v>2920</v>
+        <v>2924</v>
       </c>
       <c r="H998">
         <v>2</v>
       </c>
       <c r="I998" t="s">
-        <v>2921</v>
+        <v>2925</v>
       </c>
       <c r="J998" t="s">
         <v>2218</v>
@@ -50181,34 +50193,34 @@
     </row>
     <row r="999" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A999" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B999" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C999" t="s">
-        <v>2922</v>
+        <v>2926</v>
       </c>
       <c r="D999" t="s">
-        <v>2923</v>
+        <v>2927</v>
       </c>
       <c r="E999" t="s">
         <v>16</v>
       </c>
       <c r="F999" t="s">
-        <v>2924</v>
+        <v>2928</v>
       </c>
       <c r="G999" t="s">
-        <v>2925</v>
+        <v>2929</v>
       </c>
       <c r="H999">
         <v>2</v>
       </c>
       <c r="I999" t="s">
-        <v>2926</v>
+        <v>2930</v>
       </c>
       <c r="J999" t="s">
-        <v>2927</v>
+        <v>2931</v>
       </c>
       <c r="K999" t="s">
         <v>21</v>
@@ -50222,25 +50234,25 @@
     </row>
     <row r="1000" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1000" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1000" t="s">
-        <v>2928</v>
+        <v>2932</v>
       </c>
       <c r="D1000" t="s">
-        <v>2929</v>
+        <v>2933</v>
       </c>
       <c r="E1000" t="s">
         <v>16</v>
       </c>
       <c r="F1000" t="s">
-        <v>2930</v>
+        <v>2934</v>
       </c>
       <c r="G1000" t="s">
-        <v>2931</v>
+        <v>2935</v>
       </c>
       <c r="H1000">
         <v>2</v>
@@ -50255,7 +50267,7 @@
         <v>21</v>
       </c>
       <c r="L1000" t="s">
-        <v>2932</v>
+        <v>2936</v>
       </c>
       <c r="M1000" t="s">
         <v>23</v>
@@ -50263,31 +50275,31 @@
     </row>
     <row r="1001" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1001" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1001" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1001" t="s">
-        <v>2928</v>
+        <v>2932</v>
       </c>
       <c r="D1001" t="s">
-        <v>2929</v>
+        <v>2933</v>
       </c>
       <c r="E1001" t="s">
         <v>16</v>
       </c>
       <c r="F1001" t="s">
-        <v>2933</v>
+        <v>2937</v>
       </c>
       <c r="G1001" t="s">
-        <v>2934</v>
+        <v>2938</v>
       </c>
       <c r="H1001">
         <v>2</v>
       </c>
       <c r="I1001" t="s">
-        <v>2935</v>
+        <v>2939</v>
       </c>
       <c r="J1001" t="s">
         <v>2209</v>
@@ -50304,34 +50316,34 @@
     </row>
     <row r="1002" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1002" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1002" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1002" t="s">
-        <v>2928</v>
+        <v>2932</v>
       </c>
       <c r="D1002" t="s">
-        <v>2929</v>
+        <v>2933</v>
       </c>
       <c r="E1002" t="s">
         <v>16</v>
       </c>
       <c r="F1002" t="s">
-        <v>2936</v>
+        <v>2940</v>
       </c>
       <c r="G1002" t="s">
-        <v>2937</v>
+        <v>2941</v>
       </c>
       <c r="H1002">
         <v>2</v>
       </c>
       <c r="I1002" t="s">
-        <v>2938</v>
+        <v>2942</v>
       </c>
       <c r="J1002" t="s">
-        <v>2927</v>
+        <v>2931</v>
       </c>
       <c r="K1002" t="s">
         <v>21</v>
@@ -50345,31 +50357,31 @@
     </row>
     <row r="1003" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1003" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1003" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1003" t="s">
-        <v>2928</v>
+        <v>2932</v>
       </c>
       <c r="D1003" t="s">
-        <v>2929</v>
+        <v>2933</v>
       </c>
       <c r="E1003" t="s">
         <v>16</v>
       </c>
       <c r="F1003" t="s">
-        <v>2939</v>
+        <v>2943</v>
       </c>
       <c r="G1003" t="s">
-        <v>2940</v>
+        <v>2944</v>
       </c>
       <c r="H1003">
         <v>2</v>
       </c>
       <c r="I1003" t="s">
-        <v>2941</v>
+        <v>2945</v>
       </c>
       <c r="J1003" t="s">
         <v>1779</v>
@@ -50378,7 +50390,7 @@
         <v>21</v>
       </c>
       <c r="L1003" t="s">
-        <v>2942</v>
+        <v>2946</v>
       </c>
       <c r="M1003" t="s">
         <v>23</v>
@@ -50386,34 +50398,34 @@
     </row>
     <row r="1004" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1004" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1004" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1004" t="s">
-        <v>2943</v>
+        <v>2947</v>
       </c>
       <c r="D1004" t="s">
-        <v>2944</v>
+        <v>2948</v>
       </c>
       <c r="E1004" t="s">
         <v>16</v>
       </c>
       <c r="F1004" t="s">
-        <v>2945</v>
+        <v>2949</v>
       </c>
       <c r="G1004" t="s">
-        <v>2946</v>
+        <v>2950</v>
       </c>
       <c r="H1004">
         <v>2</v>
       </c>
       <c r="I1004" t="s">
-        <v>2947</v>
+        <v>2951</v>
       </c>
       <c r="J1004" t="s">
-        <v>2948</v>
+        <v>2952</v>
       </c>
       <c r="K1004" t="s">
         <v>21</v>
@@ -50427,31 +50439,31 @@
     </row>
     <row r="1005" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1005" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1005" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1005" t="s">
-        <v>2943</v>
+        <v>2947</v>
       </c>
       <c r="D1005" t="s">
-        <v>2944</v>
+        <v>2948</v>
       </c>
       <c r="E1005" t="s">
         <v>16</v>
       </c>
       <c r="F1005" t="s">
-        <v>2949</v>
+        <v>2953</v>
       </c>
       <c r="G1005" t="s">
-        <v>2950</v>
+        <v>2954</v>
       </c>
       <c r="H1005">
         <v>2</v>
       </c>
       <c r="I1005" t="s">
-        <v>2947</v>
+        <v>2951</v>
       </c>
       <c r="J1005" t="s">
         <v>1721</v>
@@ -50460,7 +50472,7 @@
         <v>21</v>
       </c>
       <c r="L1005" t="s">
-        <v>2942</v>
+        <v>2946</v>
       </c>
       <c r="M1005" t="s">
         <v>23</v>
@@ -50468,34 +50480,34 @@
     </row>
     <row r="1006" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1006" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1006" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1006" t="s">
-        <v>2943</v>
+        <v>2947</v>
       </c>
       <c r="D1006" t="s">
-        <v>2944</v>
+        <v>2948</v>
       </c>
       <c r="E1006" t="s">
         <v>16</v>
       </c>
       <c r="F1006" t="s">
-        <v>2951</v>
+        <v>2955</v>
       </c>
       <c r="G1006" t="s">
-        <v>2952</v>
+        <v>2956</v>
       </c>
       <c r="H1006">
         <v>2</v>
       </c>
       <c r="I1006" t="s">
-        <v>2921</v>
+        <v>2925</v>
       </c>
       <c r="J1006" t="s">
-        <v>2953</v>
+        <v>2957</v>
       </c>
       <c r="K1006" t="s">
         <v>21</v>
@@ -50509,31 +50521,31 @@
     </row>
     <row r="1007" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1007" t="s">
-        <v>2917</v>
+        <v>2921</v>
       </c>
       <c r="B1007" t="s">
-        <v>2918</v>
+        <v>2922</v>
       </c>
       <c r="C1007" t="s">
-        <v>2943</v>
+        <v>2947</v>
       </c>
       <c r="D1007" t="s">
-        <v>2944</v>
+        <v>2948</v>
       </c>
       <c r="E1007" t="s">
         <v>16</v>
       </c>
       <c r="F1007" t="s">
-        <v>2954</v>
+        <v>2958</v>
       </c>
       <c r="G1007" t="s">
-        <v>2955</v>
+        <v>2959</v>
       </c>
       <c r="H1007">
         <v>2</v>
       </c>
       <c r="I1007" t="s">
-        <v>2956</v>
+        <v>2960</v>
       </c>
       <c r="J1007" t="s">
         <v>2209</v>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-09-03T23:28Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -2089,6 +2089,9 @@
     <t>김성혜</t>
   </si>
   <si>
+    <t>월 09:00-11:00</t>
+  </si>
+  <si>
     <t>예술관3층3호실</t>
   </si>
   <si>
@@ -2135,9 +2138,6 @@
   </si>
   <si>
     <t>연효정</t>
-  </si>
-  <si>
-    <t>월 09:00-11:00</t>
   </si>
   <si>
     <t>예술관5층4호실</t>
@@ -15154,7 +15154,7 @@
         <v>21</v>
       </c>
       <c r="L128" t="s">
-        <v>164</v>
+        <v>519</v>
       </c>
       <c r="M128" t="s">
         <v>23</v>
@@ -17280,13 +17280,13 @@
         <v>691</v>
       </c>
       <c r="J180" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="K180" t="s">
         <v>21</v>
       </c>
       <c r="L180" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="M180" t="s">
         <v>643</v>
@@ -17391,16 +17391,16 @@
         <v>52</v>
       </c>
       <c r="F183" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G183" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="H183">
         <v>2</v>
       </c>
       <c r="I183" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="J183" t="s">
         <v>669</v>
@@ -17409,7 +17409,7 @@
         <v>21</v>
       </c>
       <c r="L183" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M183" t="s">
         <v>23</v>
@@ -17432,25 +17432,25 @@
         <v>52</v>
       </c>
       <c r="F184" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G184" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="H184">
         <v>2</v>
       </c>
       <c r="I184" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J184" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="K184" t="s">
         <v>21</v>
       </c>
       <c r="L184" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M184" t="s">
         <v>640</v>
@@ -17473,25 +17473,25 @@
         <v>52</v>
       </c>
       <c r="F185" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G185" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H185">
         <v>2</v>
       </c>
       <c r="I185" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J185" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="K185" t="s">
         <v>21</v>
       </c>
       <c r="L185" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M185" t="s">
         <v>23</v>
@@ -17514,25 +17514,25 @@
         <v>52</v>
       </c>
       <c r="F186" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G186" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H186">
         <v>2</v>
       </c>
       <c r="I186" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="J186" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="K186" t="s">
         <v>21</v>
       </c>
       <c r="L186" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M186" t="s">
         <v>640</v>
@@ -17555,25 +17555,25 @@
         <v>52</v>
       </c>
       <c r="F187" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G187" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H187">
         <v>2</v>
       </c>
       <c r="I187" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J187" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="K187" t="s">
         <v>21</v>
       </c>
       <c r="L187" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M187" t="s">
         <v>643</v>
@@ -17596,25 +17596,25 @@
         <v>52</v>
       </c>
       <c r="F188" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G188" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H188">
         <v>2</v>
       </c>
       <c r="I188" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J188" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="K188" t="s">
         <v>21</v>
       </c>
       <c r="L188" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M188" t="s">
         <v>646</v>
@@ -17637,19 +17637,19 @@
         <v>52</v>
       </c>
       <c r="F189" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G189" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H189">
         <v>2</v>
       </c>
       <c r="I189" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="J189" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
       <c r="K189" t="s">
         <v>21</v>
@@ -17678,16 +17678,16 @@
         <v>52</v>
       </c>
       <c r="F190" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G190" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H190">
         <v>2</v>
       </c>
       <c r="I190" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J190" t="s">
         <v>710</v>
@@ -17696,7 +17696,7 @@
         <v>21</v>
       </c>
       <c r="L190" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M190" t="s">
         <v>651</v>
@@ -17719,16 +17719,16 @@
         <v>52</v>
       </c>
       <c r="F191" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G191" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H191">
         <v>2</v>
       </c>
       <c r="I191" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J191" t="s">
         <v>711</v>
@@ -17737,7 +17737,7 @@
         <v>21</v>
       </c>
       <c r="L191" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M191" t="s">
         <v>652</v>
@@ -17778,7 +17778,7 @@
         <v>21</v>
       </c>
       <c r="L192" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M192" t="s">
         <v>23</v>
@@ -18999,7 +18999,7 @@
         <v>1</v>
       </c>
       <c r="I222" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J222" t="s">
         <v>754</v>
@@ -19008,7 +19008,7 @@
         <v>21</v>
       </c>
       <c r="L222" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M222" t="s">
         <v>23</v>
@@ -19040,7 +19040,7 @@
         <v>1</v>
       </c>
       <c r="I223" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J223" t="s">
         <v>763</v>
@@ -19049,7 +19049,7 @@
         <v>21</v>
       </c>
       <c r="L223" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M223" t="s">
         <v>640</v>
@@ -19081,7 +19081,7 @@
         <v>1</v>
       </c>
       <c r="I224" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J224" t="s">
         <v>769</v>
@@ -19090,7 +19090,7 @@
         <v>21</v>
       </c>
       <c r="L224" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M224" t="s">
         <v>643</v>
@@ -19658,7 +19658,7 @@
         <v>785</v>
       </c>
       <c r="J238" t="s">
-        <v>773</v>
+        <v>692</v>
       </c>
       <c r="K238" t="s">
         <v>21</v>
@@ -21910,7 +21910,7 @@
         <v>2</v>
       </c>
       <c r="I293" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="J293" t="s">
         <v>815</v>
@@ -21951,7 +21951,7 @@
         <v>2</v>
       </c>
       <c r="I294" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J294" t="s">
         <v>638</v>
@@ -21960,7 +21960,7 @@
         <v>21</v>
       </c>
       <c r="L294" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M294" t="s">
         <v>640</v>
@@ -21992,7 +21992,7 @@
         <v>2</v>
       </c>
       <c r="I295" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J295" t="s">
         <v>642</v>
@@ -22001,7 +22001,7 @@
         <v>21</v>
       </c>
       <c r="L295" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M295" t="s">
         <v>643</v>
@@ -22115,7 +22115,7 @@
         <v>2</v>
       </c>
       <c r="I298" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J298" t="s">
         <v>837</v>
@@ -22124,7 +22124,7 @@
         <v>21</v>
       </c>
       <c r="L298" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M298" t="s">
         <v>23</v>
@@ -22197,7 +22197,7 @@
         <v>2</v>
       </c>
       <c r="I300" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J300" t="s">
         <v>840</v>
@@ -22206,7 +22206,7 @@
         <v>21</v>
       </c>
       <c r="L300" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M300" t="s">
         <v>23</v>
@@ -22238,7 +22238,7 @@
         <v>2</v>
       </c>
       <c r="I301" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J301" t="s">
         <v>841</v>
@@ -22247,7 +22247,7 @@
         <v>21</v>
       </c>
       <c r="L301" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M301" t="s">
         <v>640</v>
@@ -22279,7 +22279,7 @@
         <v>2</v>
       </c>
       <c r="I302" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J302" t="s">
         <v>844</v>
@@ -22288,7 +22288,7 @@
         <v>21</v>
       </c>
       <c r="L302" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M302" t="s">
         <v>23</v>
@@ -22361,7 +22361,7 @@
         <v>2</v>
       </c>
       <c r="I304" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J304" t="s">
         <v>845</v>
@@ -22370,7 +22370,7 @@
         <v>21</v>
       </c>
       <c r="L304" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M304" t="s">
         <v>643</v>
@@ -22402,7 +22402,7 @@
         <v>2</v>
       </c>
       <c r="I305" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J305" t="s">
         <v>669</v>
@@ -22411,7 +22411,7 @@
         <v>21</v>
       </c>
       <c r="L305" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M305" t="s">
         <v>646</v>
@@ -22484,16 +22484,16 @@
         <v>2</v>
       </c>
       <c r="I307" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J307" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="K307" t="s">
         <v>21</v>
       </c>
       <c r="L307" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M307" t="s">
         <v>651</v>
@@ -22525,7 +22525,7 @@
         <v>2</v>
       </c>
       <c r="I308" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J308" t="s">
         <v>815</v>
@@ -22534,7 +22534,7 @@
         <v>21</v>
       </c>
       <c r="L308" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M308" t="s">
         <v>652</v>
@@ -22689,7 +22689,7 @@
         <v>3</v>
       </c>
       <c r="I312" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="J312" t="s">
         <v>854</v>
@@ -23190,7 +23190,7 @@
         <v>21</v>
       </c>
       <c r="L324" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M324" t="s">
         <v>23</v>
@@ -47462,7 +47462,7 @@
         <v>21</v>
       </c>
       <c r="L916" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="M916" t="s">
         <v>23</v>
@@ -47503,7 +47503,7 @@
         <v>21</v>
       </c>
       <c r="L917" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="M917" t="s">
         <v>23</v>
@@ -47907,7 +47907,7 @@
         <v>2854</v>
       </c>
       <c r="J927" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="K927" t="s">
         <v>21</v>
@@ -47948,7 +47948,7 @@
         <v>2858</v>
       </c>
       <c r="J928" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="K928" t="s">
         <v>21</v>
@@ -47989,7 +47989,7 @@
         <v>2861</v>
       </c>
       <c r="J929" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="K929" t="s">
         <v>21</v>
@@ -49102,7 +49102,7 @@
         <v>21</v>
       </c>
       <c r="L956" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M956" t="s">
         <v>23</v>
@@ -49143,7 +49143,7 @@
         <v>21</v>
       </c>
       <c r="L957" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M957" t="s">
         <v>640</v>
@@ -49506,7 +49506,7 @@
         <v>2961</v>
       </c>
       <c r="J966" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="K966" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-09-08T23:35Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -4528,7 +4528,7 @@
     <t>홍성지</t>
   </si>
   <si>
-    <t>월 10:00-12:00,수 10:00-12:00</t>
+    <t>월 10:30-12:00,수 10:00-12:00</t>
   </si>
   <si>
     <t>조형관별관1층1-1호실</t>
@@ -4540,7 +4540,7 @@
     <t>초급한국어2</t>
   </si>
   <si>
-    <t>화 10:00-12:00,목 10:00-12:00</t>
+    <t>화 10:30-12:00,목 10:00-12:00</t>
   </si>
   <si>
     <t>7233201</t>
@@ -30605,7 +30605,7 @@
         <v>21</v>
       </c>
       <c r="L505" t="s">
-        <v>536</v>
+        <v>580</v>
       </c>
       <c r="M505" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
feat: actions fetch kookmin 2026-09-10T23:21Z
</commit_message>
<xml_diff>
--- a/actions_fetch/out/kookmin(2026-2).xlsx
+++ b/actions_fetch/out/kookmin(2026-2).xlsx
@@ -4531,559 +4531,559 @@
     <t>월 10:30-12:00,수 10:00-12:00</t>
   </si>
   <si>
+    <t>704670a</t>
+  </si>
+  <si>
+    <t>초급한국어2</t>
+  </si>
+  <si>
+    <t>화 10:30-12:00,목 10:00-12:00</t>
+  </si>
+  <si>
+    <t>7233201</t>
+  </si>
+  <si>
+    <t>디자인 한국어1</t>
+  </si>
+  <si>
+    <t>정은주</t>
+  </si>
+  <si>
+    <t>조형관별관3층8호실</t>
+  </si>
+  <si>
+    <t>7233701</t>
+  </si>
+  <si>
+    <t>디자인 한국어2</t>
+  </si>
+  <si>
+    <t>금 09:00-13:00</t>
+  </si>
+  <si>
+    <t>조형관별관3층10호실</t>
+  </si>
+  <si>
+    <t>7233801</t>
+  </si>
+  <si>
+    <t>디자인 프랙티스2</t>
+  </si>
+  <si>
+    <t>박윤정</t>
+  </si>
+  <si>
+    <t>화 15:00-18:00,금 15:00-18:00</t>
+  </si>
+  <si>
+    <t>글로벌센터4층8호실</t>
+  </si>
+  <si>
+    <t>7233901</t>
+  </si>
+  <si>
+    <t>디자인 프랙티스1</t>
+  </si>
+  <si>
+    <t>박소영</t>
+  </si>
+  <si>
+    <t>월 15:00-18:00,목 15:00-18:00</t>
+  </si>
+  <si>
+    <t>7266001</t>
+  </si>
+  <si>
+    <t>디자인 프랙티스3</t>
+  </si>
+  <si>
+    <t>신정민</t>
+  </si>
+  <si>
+    <t>글로벌센터4층9호실</t>
+  </si>
+  <si>
+    <t>7286601</t>
+  </si>
+  <si>
+    <t>DK워크숍1</t>
+  </si>
+  <si>
+    <t>김미애</t>
+  </si>
+  <si>
+    <t>7286701</t>
+  </si>
+  <si>
+    <t>DK워크숍2</t>
+  </si>
+  <si>
+    <t>진황가</t>
+  </si>
+  <si>
+    <t>조형관별관3층7호실</t>
+  </si>
+  <si>
+    <t>36277</t>
+  </si>
+  <si>
+    <t>스마트경험디자인학과</t>
+  </si>
+  <si>
+    <t>704140b</t>
+  </si>
+  <si>
+    <t>논문ㆍ작품지도</t>
+  </si>
+  <si>
+    <t>연명흠</t>
+  </si>
+  <si>
+    <t>수 18:55-21:35</t>
+  </si>
+  <si>
+    <t>조형관별관1층5호실</t>
+  </si>
+  <si>
+    <t>704150a</t>
+  </si>
+  <si>
+    <t>논문지도1</t>
+  </si>
+  <si>
+    <t>목 18:55-21:35</t>
+  </si>
+  <si>
+    <t>조형관별관3층4호실</t>
+  </si>
+  <si>
+    <t>704160a</t>
+  </si>
+  <si>
+    <t>논문지도2</t>
+  </si>
+  <si>
+    <t>임진호</t>
+  </si>
+  <si>
+    <t>조형관별관3층5호실</t>
+  </si>
+  <si>
+    <t>689070a</t>
+  </si>
+  <si>
+    <t>인터랙션디자인2</t>
+  </si>
+  <si>
+    <t>김수진</t>
+  </si>
+  <si>
+    <t>조형관별관3층3호실</t>
+  </si>
+  <si>
+    <t>689430a</t>
+  </si>
+  <si>
+    <t>서비스디자인2</t>
+  </si>
+  <si>
+    <t>정진열</t>
+  </si>
+  <si>
+    <t>화 18:55-21:35</t>
+  </si>
+  <si>
+    <t>696070a</t>
+  </si>
+  <si>
+    <t>디자인조사분석연습</t>
+  </si>
+  <si>
+    <t>조형관별관3층2호실</t>
+  </si>
+  <si>
+    <t>스튜디오</t>
+  </si>
+  <si>
+    <t>7204501</t>
+  </si>
+  <si>
+    <t>로컬플래닝 스튜디오 2</t>
+  </si>
+  <si>
+    <t>토 10:00-16:00</t>
+  </si>
+  <si>
+    <t>7204601</t>
+  </si>
+  <si>
+    <t>기술융합디자인논제 2</t>
+  </si>
+  <si>
+    <t>정치훈</t>
+  </si>
+  <si>
+    <t>7219501</t>
+  </si>
+  <si>
+    <t>도시공간론2</t>
+  </si>
+  <si>
+    <t>이용원</t>
+  </si>
+  <si>
+    <t>월 18:55-21:35</t>
+  </si>
+  <si>
+    <t>7231401</t>
+  </si>
+  <si>
+    <t>인공지능 활용 디자인</t>
+  </si>
+  <si>
+    <t>7244101</t>
+  </si>
+  <si>
+    <t>AI-XR 디자인</t>
+  </si>
+  <si>
+    <t>한주현</t>
+  </si>
+  <si>
+    <t>7249001</t>
+  </si>
+  <si>
+    <t>로컬혁신세미나2</t>
+  </si>
+  <si>
+    <t>7253701</t>
+  </si>
+  <si>
+    <t>기후변화와 서비스디자인</t>
+  </si>
+  <si>
+    <t>유채문</t>
+  </si>
+  <si>
+    <t>7260501</t>
+  </si>
+  <si>
+    <t>인클루시브 디자인</t>
+  </si>
+  <si>
+    <t>7286301</t>
+  </si>
+  <si>
+    <t>인간-인공지능 협업디자인 스튜디오2</t>
+  </si>
+  <si>
+    <t>허정윤</t>
+  </si>
+  <si>
+    <t>월 14:00-17:00,수 10:00-13:00</t>
+  </si>
+  <si>
+    <t>조형관별관3층10호실,조형관별관3층2호실</t>
+  </si>
+  <si>
+    <t>7295401</t>
+  </si>
+  <si>
+    <t>AI콘텐츠디자인스튜디오1</t>
+  </si>
+  <si>
+    <t>권주영</t>
+  </si>
+  <si>
+    <t>월 14:00-19:45</t>
+  </si>
+  <si>
+    <t>김진영</t>
+  </si>
+  <si>
+    <t>월 10:00-13:00,목 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7295501</t>
+  </si>
+  <si>
+    <t>AI 시대의 인간이해</t>
+  </si>
+  <si>
+    <t>7295601</t>
+  </si>
+  <si>
+    <t>Agentic UX디자인</t>
+  </si>
+  <si>
+    <t>7295701</t>
+  </si>
+  <si>
+    <t>서비스디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>조만수</t>
+  </si>
+  <si>
+    <t>월 10:00-13:00,수 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7295901</t>
+  </si>
+  <si>
+    <t>사운드경험디자인</t>
+  </si>
+  <si>
+    <t>남궁기찬</t>
+  </si>
+  <si>
+    <t>월 11:00-14:00</t>
+  </si>
+  <si>
+    <t>7296001</t>
+  </si>
+  <si>
+    <t>제품서비스시스템디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>심유리</t>
+  </si>
+  <si>
+    <t>월 10:00-17:00</t>
+  </si>
+  <si>
+    <t>7296101</t>
+  </si>
+  <si>
+    <t>정보디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>허정현</t>
+  </si>
+  <si>
+    <t>월 18:00-20:40,수 14:30-17:30</t>
+  </si>
+  <si>
+    <t>조형관별관3층3호실,조형관별관3층10호실</t>
+  </si>
+  <si>
+    <t>7296201</t>
+  </si>
+  <si>
+    <t>공공서비스디자인</t>
+  </si>
+  <si>
+    <t>박순정</t>
+  </si>
+  <si>
+    <t>조형관별관3층9호실</t>
+  </si>
+  <si>
+    <t>7296301</t>
+  </si>
+  <si>
+    <t>정량연구방법</t>
+  </si>
+  <si>
+    <t>36320</t>
+  </si>
+  <si>
+    <t>공간ㆍ문화디자인학과</t>
+  </si>
+  <si>
+    <t>704200b</t>
+  </si>
+  <si>
+    <t>7243701</t>
+  </si>
+  <si>
+    <t>특수연구과제2</t>
+  </si>
+  <si>
+    <t>윤성호</t>
+  </si>
+  <si>
+    <t>조형관별관3층14호실</t>
+  </si>
+  <si>
+    <t>7294501</t>
+  </si>
+  <si>
+    <t>7295101</t>
+  </si>
+  <si>
+    <t>강민선</t>
+  </si>
+  <si>
+    <t>707590a</t>
+  </si>
+  <si>
+    <t>소재 융합 개발 연구</t>
+  </si>
+  <si>
+    <t>이순정</t>
+  </si>
+  <si>
+    <t>토 10:00-13:00</t>
+  </si>
+  <si>
+    <t>7129001</t>
+  </si>
+  <si>
+    <t>디자인리서치&amp;방법론</t>
+  </si>
+  <si>
+    <t>7192201</t>
+  </si>
+  <si>
+    <t>글로벌 디자인 워크샵</t>
+  </si>
+  <si>
+    <t>정상엽</t>
+  </si>
+  <si>
+    <t>7192301</t>
+  </si>
+  <si>
+    <t>공간디자인 리서치 1</t>
+  </si>
+  <si>
+    <t>고은주</t>
+  </si>
+  <si>
+    <t>7243801</t>
+  </si>
+  <si>
+    <t>현대도시디자인</t>
+  </si>
+  <si>
+    <t>김상호</t>
+  </si>
+  <si>
+    <t>7262401</t>
+  </si>
+  <si>
+    <t>사진과 문화공간</t>
+  </si>
+  <si>
+    <t>김규랑</t>
+  </si>
+  <si>
+    <t>7294101</t>
+  </si>
+  <si>
+    <t>미래디자인트렌드</t>
+  </si>
+  <si>
+    <t>박성미</t>
+  </si>
+  <si>
+    <t>7294201</t>
+  </si>
+  <si>
+    <t>리빙제품 및 신소재연구</t>
+  </si>
+  <si>
+    <t>7294301</t>
+  </si>
+  <si>
+    <t>리빙 및 가구 제품 기획</t>
+  </si>
+  <si>
+    <t>김상현</t>
+  </si>
+  <si>
+    <t>토 13:00-18:50</t>
+  </si>
+  <si>
+    <t>7294401</t>
+  </si>
+  <si>
+    <t>융합실내디자인스튜디오1</t>
+  </si>
+  <si>
+    <t>7294601</t>
+  </si>
+  <si>
+    <t>문화현장리서치</t>
+  </si>
+  <si>
+    <t>이상해</t>
+  </si>
+  <si>
+    <t>7294701</t>
+  </si>
+  <si>
+    <t>디지털공간디자인1</t>
+  </si>
+  <si>
+    <t>민세희</t>
+  </si>
+  <si>
+    <t>7294801</t>
+  </si>
+  <si>
+    <t>융합공간디자인세미나</t>
+  </si>
+  <si>
+    <t>7294901</t>
+  </si>
+  <si>
+    <t>인터렉티브 환경디자인 스튜디오1</t>
+  </si>
+  <si>
+    <t>7295001</t>
+  </si>
+  <si>
+    <t>공간디자인스튜디오2</t>
+  </si>
+  <si>
+    <t>7295201</t>
+  </si>
+  <si>
+    <t>크리에이티브스페이스스튜디오1</t>
+  </si>
+  <si>
+    <t>7295301</t>
+  </si>
+  <si>
+    <t>뉴미디어환경디자인스튜디오1</t>
+  </si>
+  <si>
+    <t>36378</t>
+  </si>
+  <si>
+    <t>융합디자인학과</t>
+  </si>
+  <si>
+    <t>689540b</t>
+  </si>
+  <si>
+    <t>성재혁</t>
+  </si>
+  <si>
+    <t>689260a</t>
+  </si>
+  <si>
+    <t>704700a</t>
+  </si>
+  <si>
+    <t>사회적책임과디자인4</t>
+  </si>
+  <si>
+    <t>최호랑</t>
+  </si>
+  <si>
+    <t>7130201</t>
+  </si>
+  <si>
+    <t>타이포그래픽 디자인4</t>
+  </si>
+  <si>
+    <t>화 10:00-13:00,금 10:00-13:00</t>
+  </si>
+  <si>
     <t>조형관별관1층1-1호실</t>
-  </si>
-  <si>
-    <t>704670a</t>
-  </si>
-  <si>
-    <t>초급한국어2</t>
-  </si>
-  <si>
-    <t>화 10:30-12:00,목 10:00-12:00</t>
-  </si>
-  <si>
-    <t>7233201</t>
-  </si>
-  <si>
-    <t>디자인 한국어1</t>
-  </si>
-  <si>
-    <t>정은주</t>
-  </si>
-  <si>
-    <t>조형관별관3층8호실</t>
-  </si>
-  <si>
-    <t>7233701</t>
-  </si>
-  <si>
-    <t>디자인 한국어2</t>
-  </si>
-  <si>
-    <t>금 09:00-13:00</t>
-  </si>
-  <si>
-    <t>7233801</t>
-  </si>
-  <si>
-    <t>디자인 프랙티스2</t>
-  </si>
-  <si>
-    <t>박윤정</t>
-  </si>
-  <si>
-    <t>화 15:00-18:00,금 15:00-18:00</t>
-  </si>
-  <si>
-    <t>글로벌센터4층8호실</t>
-  </si>
-  <si>
-    <t>7233901</t>
-  </si>
-  <si>
-    <t>디자인 프랙티스1</t>
-  </si>
-  <si>
-    <t>박소영</t>
-  </si>
-  <si>
-    <t>월 15:00-18:00,목 15:00-18:00</t>
-  </si>
-  <si>
-    <t>7266001</t>
-  </si>
-  <si>
-    <t>디자인 프랙티스3</t>
-  </si>
-  <si>
-    <t>신정민</t>
-  </si>
-  <si>
-    <t>글로벌센터4층9호실</t>
-  </si>
-  <si>
-    <t>7286601</t>
-  </si>
-  <si>
-    <t>DK워크숍1</t>
-  </si>
-  <si>
-    <t>김미애</t>
-  </si>
-  <si>
-    <t>7286701</t>
-  </si>
-  <si>
-    <t>DK워크숍2</t>
-  </si>
-  <si>
-    <t>진황가</t>
-  </si>
-  <si>
-    <t>조형관별관3층7호실</t>
-  </si>
-  <si>
-    <t>36277</t>
-  </si>
-  <si>
-    <t>스마트경험디자인학과</t>
-  </si>
-  <si>
-    <t>704140b</t>
-  </si>
-  <si>
-    <t>논문ㆍ작품지도</t>
-  </si>
-  <si>
-    <t>연명흠</t>
-  </si>
-  <si>
-    <t>수 18:55-21:35</t>
-  </si>
-  <si>
-    <t>조형관별관1층5호실</t>
-  </si>
-  <si>
-    <t>704150a</t>
-  </si>
-  <si>
-    <t>논문지도1</t>
-  </si>
-  <si>
-    <t>목 18:55-21:35</t>
-  </si>
-  <si>
-    <t>조형관별관3층4호실</t>
-  </si>
-  <si>
-    <t>704160a</t>
-  </si>
-  <si>
-    <t>논문지도2</t>
-  </si>
-  <si>
-    <t>임진호</t>
-  </si>
-  <si>
-    <t>조형관별관3층5호실</t>
-  </si>
-  <si>
-    <t>689070a</t>
-  </si>
-  <si>
-    <t>인터랙션디자인2</t>
-  </si>
-  <si>
-    <t>김수진</t>
-  </si>
-  <si>
-    <t>조형관별관3층3호실</t>
-  </si>
-  <si>
-    <t>689430a</t>
-  </si>
-  <si>
-    <t>서비스디자인2</t>
-  </si>
-  <si>
-    <t>정진열</t>
-  </si>
-  <si>
-    <t>화 18:55-21:35</t>
-  </si>
-  <si>
-    <t>696070a</t>
-  </si>
-  <si>
-    <t>디자인조사분석연습</t>
-  </si>
-  <si>
-    <t>조형관별관3층2호실</t>
-  </si>
-  <si>
-    <t>스튜디오</t>
-  </si>
-  <si>
-    <t>7204501</t>
-  </si>
-  <si>
-    <t>로컬플래닝 스튜디오 2</t>
-  </si>
-  <si>
-    <t>토 10:00-16:00</t>
-  </si>
-  <si>
-    <t>7204601</t>
-  </si>
-  <si>
-    <t>기술융합디자인논제 2</t>
-  </si>
-  <si>
-    <t>정치훈</t>
-  </si>
-  <si>
-    <t>7219501</t>
-  </si>
-  <si>
-    <t>도시공간론2</t>
-  </si>
-  <si>
-    <t>이용원</t>
-  </si>
-  <si>
-    <t>월 18:55-21:35</t>
-  </si>
-  <si>
-    <t>7231401</t>
-  </si>
-  <si>
-    <t>인공지능 활용 디자인</t>
-  </si>
-  <si>
-    <t>7244101</t>
-  </si>
-  <si>
-    <t>AI-XR 디자인</t>
-  </si>
-  <si>
-    <t>한주현</t>
-  </si>
-  <si>
-    <t>7249001</t>
-  </si>
-  <si>
-    <t>로컬혁신세미나2</t>
-  </si>
-  <si>
-    <t>7253701</t>
-  </si>
-  <si>
-    <t>기후변화와 서비스디자인</t>
-  </si>
-  <si>
-    <t>유채문</t>
-  </si>
-  <si>
-    <t>7260501</t>
-  </si>
-  <si>
-    <t>인클루시브 디자인</t>
-  </si>
-  <si>
-    <t>조형관별관3층10호실</t>
-  </si>
-  <si>
-    <t>7286301</t>
-  </si>
-  <si>
-    <t>인간-인공지능 협업디자인 스튜디오2</t>
-  </si>
-  <si>
-    <t>허정윤</t>
-  </si>
-  <si>
-    <t>월 14:00-17:00,수 10:00-13:00</t>
-  </si>
-  <si>
-    <t>조형관별관3층10호실,조형관별관3층2호실</t>
-  </si>
-  <si>
-    <t>7295401</t>
-  </si>
-  <si>
-    <t>AI콘텐츠디자인스튜디오1</t>
-  </si>
-  <si>
-    <t>권주영</t>
-  </si>
-  <si>
-    <t>월 14:00-19:45</t>
-  </si>
-  <si>
-    <t>김진영</t>
-  </si>
-  <si>
-    <t>월 10:00-13:00,목 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7295501</t>
-  </si>
-  <si>
-    <t>AI 시대의 인간이해</t>
-  </si>
-  <si>
-    <t>7295601</t>
-  </si>
-  <si>
-    <t>Agentic UX디자인</t>
-  </si>
-  <si>
-    <t>7295701</t>
-  </si>
-  <si>
-    <t>서비스디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>조만수</t>
-  </si>
-  <si>
-    <t>월 10:00-13:00,수 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7295901</t>
-  </si>
-  <si>
-    <t>사운드경험디자인</t>
-  </si>
-  <si>
-    <t>남궁기찬</t>
-  </si>
-  <si>
-    <t>월 11:00-14:00</t>
-  </si>
-  <si>
-    <t>7296001</t>
-  </si>
-  <si>
-    <t>제품서비스시스템디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>심유리</t>
-  </si>
-  <si>
-    <t>월 10:00-17:00</t>
-  </si>
-  <si>
-    <t>7296101</t>
-  </si>
-  <si>
-    <t>정보디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>허정현</t>
-  </si>
-  <si>
-    <t>월 18:00-20:40,수 14:30-17:30</t>
-  </si>
-  <si>
-    <t>조형관별관3층3호실,조형관별관3층10호실</t>
-  </si>
-  <si>
-    <t>7296201</t>
-  </si>
-  <si>
-    <t>공공서비스디자인</t>
-  </si>
-  <si>
-    <t>박순정</t>
-  </si>
-  <si>
-    <t>조형관별관3층9호실</t>
-  </si>
-  <si>
-    <t>7296301</t>
-  </si>
-  <si>
-    <t>정량연구방법</t>
-  </si>
-  <si>
-    <t>36320</t>
-  </si>
-  <si>
-    <t>공간ㆍ문화디자인학과</t>
-  </si>
-  <si>
-    <t>704200b</t>
-  </si>
-  <si>
-    <t>7243701</t>
-  </si>
-  <si>
-    <t>특수연구과제2</t>
-  </si>
-  <si>
-    <t>윤성호</t>
-  </si>
-  <si>
-    <t>조형관별관3층14호실</t>
-  </si>
-  <si>
-    <t>7294501</t>
-  </si>
-  <si>
-    <t>7295101</t>
-  </si>
-  <si>
-    <t>강민선</t>
-  </si>
-  <si>
-    <t>707590a</t>
-  </si>
-  <si>
-    <t>소재 융합 개발 연구</t>
-  </si>
-  <si>
-    <t>이순정</t>
-  </si>
-  <si>
-    <t>토 10:00-13:00</t>
-  </si>
-  <si>
-    <t>7129001</t>
-  </si>
-  <si>
-    <t>디자인리서치&amp;방법론</t>
-  </si>
-  <si>
-    <t>7192201</t>
-  </si>
-  <si>
-    <t>글로벌 디자인 워크샵</t>
-  </si>
-  <si>
-    <t>정상엽</t>
-  </si>
-  <si>
-    <t>7192301</t>
-  </si>
-  <si>
-    <t>공간디자인 리서치 1</t>
-  </si>
-  <si>
-    <t>고은주</t>
-  </si>
-  <si>
-    <t>7243801</t>
-  </si>
-  <si>
-    <t>현대도시디자인</t>
-  </si>
-  <si>
-    <t>김상호</t>
-  </si>
-  <si>
-    <t>7262401</t>
-  </si>
-  <si>
-    <t>사진과 문화공간</t>
-  </si>
-  <si>
-    <t>김규랑</t>
-  </si>
-  <si>
-    <t>7294101</t>
-  </si>
-  <si>
-    <t>미래디자인트렌드</t>
-  </si>
-  <si>
-    <t>박성미</t>
-  </si>
-  <si>
-    <t>7294201</t>
-  </si>
-  <si>
-    <t>리빙제품 및 신소재연구</t>
-  </si>
-  <si>
-    <t>7294301</t>
-  </si>
-  <si>
-    <t>리빙 및 가구 제품 기획</t>
-  </si>
-  <si>
-    <t>김상현</t>
-  </si>
-  <si>
-    <t>토 13:00-18:50</t>
-  </si>
-  <si>
-    <t>7294401</t>
-  </si>
-  <si>
-    <t>융합실내디자인스튜디오1</t>
-  </si>
-  <si>
-    <t>7294601</t>
-  </si>
-  <si>
-    <t>문화현장리서치</t>
-  </si>
-  <si>
-    <t>이상해</t>
-  </si>
-  <si>
-    <t>7294701</t>
-  </si>
-  <si>
-    <t>디지털공간디자인1</t>
-  </si>
-  <si>
-    <t>민세희</t>
-  </si>
-  <si>
-    <t>7294801</t>
-  </si>
-  <si>
-    <t>융합공간디자인세미나</t>
-  </si>
-  <si>
-    <t>7294901</t>
-  </si>
-  <si>
-    <t>인터렉티브 환경디자인 스튜디오1</t>
-  </si>
-  <si>
-    <t>7295001</t>
-  </si>
-  <si>
-    <t>공간디자인스튜디오2</t>
-  </si>
-  <si>
-    <t>7295201</t>
-  </si>
-  <si>
-    <t>크리에이티브스페이스스튜디오1</t>
-  </si>
-  <si>
-    <t>7295301</t>
-  </si>
-  <si>
-    <t>뉴미디어환경디자인스튜디오1</t>
-  </si>
-  <si>
-    <t>36378</t>
-  </si>
-  <si>
-    <t>융합디자인학과</t>
-  </si>
-  <si>
-    <t>689540b</t>
-  </si>
-  <si>
-    <t>성재혁</t>
-  </si>
-  <si>
-    <t>689260a</t>
-  </si>
-  <si>
-    <t>704700a</t>
-  </si>
-  <si>
-    <t>사회적책임과디자인4</t>
-  </si>
-  <si>
-    <t>최호랑</t>
-  </si>
-  <si>
-    <t>7130201</t>
-  </si>
-  <si>
-    <t>타이포그래픽 디자인4</t>
-  </si>
-  <si>
-    <t>화 10:00-13:00,금 10:00-13:00</t>
   </si>
   <si>
     <t>7231901</t>
@@ -30564,7 +30564,7 @@
         <v>21</v>
       </c>
       <c r="L504" t="s">
-        <v>1506</v>
+        <v>536</v>
       </c>
       <c r="M504" t="s">
         <v>23</v>
@@ -30587,10 +30587,10 @@
         <v>1501</v>
       </c>
       <c r="F505" t="s">
+        <v>1506</v>
+      </c>
+      <c r="G505" t="s">
         <v>1507</v>
-      </c>
-      <c r="G505" t="s">
-        <v>1508</v>
       </c>
       <c r="H505">
         <v>3</v>
@@ -30599,7 +30599,7 @@
         <v>1504</v>
       </c>
       <c r="J505" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="K505" t="s">
         <v>21</v>
@@ -30628,16 +30628,16 @@
         <v>1501</v>
       </c>
       <c r="F506" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G506" t="s">
         <v>1510</v>
       </c>
-      <c r="G506" t="s">
+      <c r="H506">
+        <v>3</v>
+      </c>
+      <c r="I506" t="s">
         <v>1511</v>
-      </c>
-      <c r="H506">
-        <v>3</v>
-      </c>
-      <c r="I506" t="s">
-        <v>1512</v>
       </c>
       <c r="J506" t="s">
         <v>531</v>
@@ -30646,7 +30646,7 @@
         <v>21</v>
       </c>
       <c r="L506" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M506" t="s">
         <v>23</v>
@@ -30669,25 +30669,25 @@
         <v>1501</v>
       </c>
       <c r="F507" t="s">
+        <v>1513</v>
+      </c>
+      <c r="G507" t="s">
         <v>1514</v>
       </c>
-      <c r="G507" t="s">
+      <c r="H507">
+        <v>3</v>
+      </c>
+      <c r="I507" t="s">
+        <v>1511</v>
+      </c>
+      <c r="J507" t="s">
         <v>1515</v>
       </c>
-      <c r="H507">
-        <v>3</v>
-      </c>
-      <c r="I507" t="s">
-        <v>1512</v>
-      </c>
-      <c r="J507" t="s">
+      <c r="K507" t="s">
+        <v>21</v>
+      </c>
+      <c r="L507" t="s">
         <v>1516</v>
-      </c>
-      <c r="K507" t="s">
-        <v>21</v>
-      </c>
-      <c r="L507" t="s">
-        <v>1513</v>
       </c>
       <c r="M507" t="s">
         <v>23</v>
@@ -30851,7 +30851,7 @@
         <v>21</v>
       </c>
       <c r="L511" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M511" t="s">
         <v>23</v>
@@ -31302,7 +31302,7 @@
         <v>21</v>
       </c>
       <c r="L522" t="s">
-        <v>1547</v>
+        <v>1562</v>
       </c>
       <c r="M522" t="s">
         <v>23</v>
@@ -31466,7 +31466,7 @@
         <v>21</v>
       </c>
       <c r="L526" t="s">
-        <v>1586</v>
+        <v>1516</v>
       </c>
       <c r="M526" t="s">
         <v>23</v>
@@ -31489,25 +31489,25 @@
         <v>1563</v>
       </c>
       <c r="F527" t="s">
+        <v>1586</v>
+      </c>
+      <c r="G527" t="s">
         <v>1587</v>
-      </c>
-      <c r="G527" t="s">
-        <v>1588</v>
       </c>
       <c r="H527">
         <v>6</v>
       </c>
       <c r="I527" t="s">
+        <v>1588</v>
+      </c>
+      <c r="J527" t="s">
         <v>1589</v>
       </c>
-      <c r="J527" t="s">
+      <c r="K527" t="s">
+        <v>21</v>
+      </c>
+      <c r="L527" t="s">
         <v>1590</v>
-      </c>
-      <c r="K527" t="s">
-        <v>21</v>
-      </c>
-      <c r="L527" t="s">
-        <v>1591</v>
       </c>
       <c r="M527" t="s">
         <v>23</v>
@@ -31530,19 +31530,19 @@
         <v>1563</v>
       </c>
       <c r="F528" t="s">
+        <v>1591</v>
+      </c>
+      <c r="G528" t="s">
         <v>1592</v>
-      </c>
-      <c r="G528" t="s">
-        <v>1593</v>
       </c>
       <c r="H528">
         <v>6</v>
       </c>
       <c r="I528" t="s">
+        <v>1593</v>
+      </c>
+      <c r="J528" t="s">
         <v>1594</v>
-      </c>
-      <c r="J528" t="s">
-        <v>1595</v>
       </c>
       <c r="K528" t="s">
         <v>21</v>
@@ -31571,19 +31571,19 @@
         <v>1563</v>
       </c>
       <c r="F529" t="s">
+        <v>1591</v>
+      </c>
+      <c r="G529" t="s">
         <v>1592</v>
-      </c>
-      <c r="G529" t="s">
-        <v>1593</v>
       </c>
       <c r="H529">
         <v>6</v>
       </c>
       <c r="I529" t="s">
+        <v>1595</v>
+      </c>
+      <c r="J529" t="s">
         <v>1596</v>
-      </c>
-      <c r="J529" t="s">
-        <v>1597</v>
       </c>
       <c r="K529" t="s">
         <v>21</v>
@@ -31612,16 +31612,16 @@
         <v>52</v>
       </c>
       <c r="F530" t="s">
+        <v>1597</v>
+      </c>
+      <c r="G530" t="s">
         <v>1598</v>
       </c>
-      <c r="G530" t="s">
-        <v>1599</v>
-      </c>
       <c r="H530">
         <v>3</v>
       </c>
       <c r="I530" t="s">
-        <v>1589</v>
+        <v>1588</v>
       </c>
       <c r="J530" t="s">
         <v>86</v>
@@ -31630,7 +31630,7 @@
         <v>21</v>
       </c>
       <c r="L530" t="s">
-        <v>1586</v>
+        <v>1516</v>
       </c>
       <c r="M530" t="s">
         <v>23</v>
@@ -31653,16 +31653,16 @@
         <v>52</v>
       </c>
       <c r="F531" t="s">
+        <v>1599</v>
+      </c>
+      <c r="G531" t="s">
         <v>1600</v>
       </c>
-      <c r="G531" t="s">
-        <v>1601</v>
-      </c>
       <c r="H531">
         <v>3</v>
       </c>
       <c r="I531" t="s">
-        <v>1589</v>
+        <v>1588</v>
       </c>
       <c r="J531" t="s">
         <v>117</v>
@@ -31671,7 +31671,7 @@
         <v>21</v>
       </c>
       <c r="L531" t="s">
-        <v>1586</v>
+        <v>1516</v>
       </c>
       <c r="M531" t="s">
         <v>23</v>
@@ -31694,19 +31694,19 @@
         <v>1563</v>
       </c>
       <c r="F532" t="s">
+        <v>1601</v>
+      </c>
+      <c r="G532" t="s">
         <v>1602</v>
-      </c>
-      <c r="G532" t="s">
-        <v>1603</v>
       </c>
       <c r="H532">
         <v>6</v>
       </c>
       <c r="I532" t="s">
+        <v>1603</v>
+      </c>
+      <c r="J532" t="s">
         <v>1604</v>
-      </c>
-      <c r="J532" t="s">
-        <v>1605</v>
       </c>
       <c r="K532" t="s">
         <v>21</v>
@@ -31735,19 +31735,19 @@
         <v>52</v>
       </c>
       <c r="F533" t="s">
+        <v>1605</v>
+      </c>
+      <c r="G533" t="s">
         <v>1606</v>
       </c>
-      <c r="G533" t="s">
+      <c r="H533">
+        <v>3</v>
+      </c>
+      <c r="I533" t="s">
         <v>1607</v>
       </c>
-      <c r="H533">
-        <v>3</v>
-      </c>
-      <c r="I533" t="s">
+      <c r="J533" t="s">
         <v>1608</v>
-      </c>
-      <c r="J533" t="s">
-        <v>1609</v>
       </c>
       <c r="K533" t="s">
         <v>21</v>
@@ -31776,19 +31776,19 @@
         <v>1563</v>
       </c>
       <c r="F534" t="s">
+        <v>1609</v>
+      </c>
+      <c r="G534" t="s">
         <v>1610</v>
-      </c>
-      <c r="G534" t="s">
-        <v>1611</v>
       </c>
       <c r="H534">
         <v>6</v>
       </c>
       <c r="I534" t="s">
+        <v>1611</v>
+      </c>
+      <c r="J534" t="s">
         <v>1612</v>
-      </c>
-      <c r="J534" t="s">
-        <v>1613</v>
       </c>
       <c r="K534" t="s">
         <v>21</v>
@@ -31817,25 +31817,25 @@
         <v>1563</v>
       </c>
       <c r="F535" t="s">
+        <v>1613</v>
+      </c>
+      <c r="G535" t="s">
         <v>1614</v>
-      </c>
-      <c r="G535" t="s">
-        <v>1615</v>
       </c>
       <c r="H535">
         <v>6</v>
       </c>
       <c r="I535" t="s">
+        <v>1615</v>
+      </c>
+      <c r="J535" t="s">
         <v>1616</v>
       </c>
-      <c r="J535" t="s">
+      <c r="K535" t="s">
+        <v>21</v>
+      </c>
+      <c r="L535" t="s">
         <v>1617</v>
-      </c>
-      <c r="K535" t="s">
-        <v>21</v>
-      </c>
-      <c r="L535" t="s">
-        <v>1618</v>
       </c>
       <c r="M535" t="s">
         <v>23</v>
@@ -31858,16 +31858,16 @@
         <v>52</v>
       </c>
       <c r="F536" t="s">
+        <v>1618</v>
+      </c>
+      <c r="G536" t="s">
         <v>1619</v>
       </c>
-      <c r="G536" t="s">
+      <c r="H536">
+        <v>3</v>
+      </c>
+      <c r="I536" t="s">
         <v>1620</v>
-      </c>
-      <c r="H536">
-        <v>3</v>
-      </c>
-      <c r="I536" t="s">
-        <v>1621</v>
       </c>
       <c r="J536" t="s">
         <v>86</v>
@@ -31876,7 +31876,7 @@
         <v>21</v>
       </c>
       <c r="L536" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="M536" t="s">
         <v>23</v>
@@ -31899,16 +31899,16 @@
         <v>52</v>
       </c>
       <c r="F537" t="s">
+        <v>1622</v>
+      </c>
+      <c r="G537" t="s">
         <v>1623</v>
       </c>
-      <c r="G537" t="s">
-        <v>1624</v>
-      </c>
       <c r="H537">
         <v>3</v>
       </c>
       <c r="I537" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="J537" t="s">
         <v>163</v>
@@ -31931,16 +31931,16 @@
         <v>1500</v>
       </c>
       <c r="C538" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D538" t="s">
         <v>1625</v>
-      </c>
-      <c r="D538" t="s">
-        <v>1626</v>
       </c>
       <c r="E538" t="s">
         <v>52</v>
       </c>
       <c r="F538" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="G538" t="s">
         <v>1540</v>
@@ -31972,25 +31972,25 @@
         <v>1500</v>
       </c>
       <c r="C539" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D539" t="s">
         <v>1625</v>
-      </c>
-      <c r="D539" t="s">
-        <v>1626</v>
       </c>
       <c r="E539" t="s">
         <v>52</v>
       </c>
       <c r="F539" t="s">
+        <v>1627</v>
+      </c>
+      <c r="G539" t="s">
         <v>1628</v>
       </c>
-      <c r="G539" t="s">
+      <c r="H539">
+        <v>3</v>
+      </c>
+      <c r="I539" t="s">
         <v>1629</v>
-      </c>
-      <c r="H539">
-        <v>3</v>
-      </c>
-      <c r="I539" t="s">
-        <v>1630</v>
       </c>
       <c r="J539" t="s">
         <v>70</v>
@@ -31999,7 +31999,7 @@
         <v>21</v>
       </c>
       <c r="L539" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="M539" t="s">
         <v>23</v>
@@ -32013,16 +32013,16 @@
         <v>1500</v>
       </c>
       <c r="C540" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D540" t="s">
         <v>1625</v>
-      </c>
-      <c r="D540" t="s">
-        <v>1626</v>
       </c>
       <c r="E540" t="s">
         <v>52</v>
       </c>
       <c r="F540" t="s">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="G540" t="s">
         <v>1549</v>
@@ -32040,7 +32040,7 @@
         <v>21</v>
       </c>
       <c r="L540" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M540" t="s">
         <v>23</v>
@@ -32054,16 +32054,16 @@
         <v>1500</v>
       </c>
       <c r="C541" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D541" t="s">
         <v>1625</v>
-      </c>
-      <c r="D541" t="s">
-        <v>1626</v>
       </c>
       <c r="E541" t="s">
         <v>52</v>
       </c>
       <c r="F541" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="G541" t="s">
         <v>1545</v>
@@ -32072,7 +32072,7 @@
         <v>3</v>
       </c>
       <c r="I541" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="J541" t="s">
         <v>359</v>
@@ -32095,34 +32095,34 @@
         <v>1500</v>
       </c>
       <c r="C542" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D542" t="s">
         <v>1625</v>
-      </c>
-      <c r="D542" t="s">
-        <v>1626</v>
       </c>
       <c r="E542" t="s">
         <v>52</v>
       </c>
       <c r="F542" t="s">
+        <v>1634</v>
+      </c>
+      <c r="G542" t="s">
         <v>1635</v>
       </c>
-      <c r="G542" t="s">
+      <c r="H542">
+        <v>3</v>
+      </c>
+      <c r="I542" t="s">
         <v>1636</v>
       </c>
-      <c r="H542">
-        <v>3</v>
-      </c>
-      <c r="I542" t="s">
+      <c r="J542" t="s">
         <v>1637</v>
       </c>
-      <c r="J542" t="s">
-        <v>1638</v>
-      </c>
       <c r="K542" t="s">
         <v>21</v>
       </c>
       <c r="L542" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="M542" t="s">
         <v>23</v>
@@ -32136,19 +32136,19 @@
         <v>1500</v>
       </c>
       <c r="C543" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D543" t="s">
         <v>1625</v>
-      </c>
-      <c r="D543" t="s">
-        <v>1626</v>
       </c>
       <c r="E543" t="s">
         <v>52</v>
       </c>
       <c r="F543" t="s">
+        <v>1638</v>
+      </c>
+      <c r="G543" t="s">
         <v>1639</v>
-      </c>
-      <c r="G543" t="s">
-        <v>1640</v>
       </c>
       <c r="H543">
         <v>3</v>
@@ -32163,7 +32163,7 @@
         <v>21</v>
       </c>
       <c r="L543" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M543" t="s">
         <v>23</v>
@@ -32177,25 +32177,25 @@
         <v>1500</v>
       </c>
       <c r="C544" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D544" t="s">
         <v>1625</v>
-      </c>
-      <c r="D544" t="s">
-        <v>1626</v>
       </c>
       <c r="E544" t="s">
         <v>1563</v>
       </c>
       <c r="F544" t="s">
+        <v>1640</v>
+      </c>
+      <c r="G544" t="s">
         <v>1641</v>
       </c>
-      <c r="G544" t="s">
+      <c r="H544">
+        <v>3</v>
+      </c>
+      <c r="I544" t="s">
         <v>1642</v>
-      </c>
-      <c r="H544">
-        <v>3</v>
-      </c>
-      <c r="I544" t="s">
-        <v>1643</v>
       </c>
       <c r="J544" t="s">
         <v>854</v>
@@ -32218,25 +32218,25 @@
         <v>1500</v>
       </c>
       <c r="C545" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D545" t="s">
         <v>1625</v>
-      </c>
-      <c r="D545" t="s">
-        <v>1626</v>
       </c>
       <c r="E545" t="s">
         <v>52</v>
       </c>
       <c r="F545" t="s">
+        <v>1643</v>
+      </c>
+      <c r="G545" t="s">
         <v>1644</v>
       </c>
-      <c r="G545" t="s">
+      <c r="H545">
+        <v>3</v>
+      </c>
+      <c r="I545" t="s">
         <v>1645</v>
-      </c>
-      <c r="H545">
-        <v>3</v>
-      </c>
-      <c r="I545" t="s">
-        <v>1646</v>
       </c>
       <c r="J545" t="s">
         <v>163</v>
@@ -32245,7 +32245,7 @@
         <v>21</v>
       </c>
       <c r="L545" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M545" t="s">
         <v>23</v>
@@ -32259,25 +32259,25 @@
         <v>1500</v>
       </c>
       <c r="C546" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D546" t="s">
         <v>1625</v>
-      </c>
-      <c r="D546" t="s">
-        <v>1626</v>
       </c>
       <c r="E546" t="s">
         <v>52</v>
       </c>
       <c r="F546" t="s">
+        <v>1646</v>
+      </c>
+      <c r="G546" t="s">
         <v>1647</v>
       </c>
-      <c r="G546" t="s">
+      <c r="H546">
+        <v>3</v>
+      </c>
+      <c r="I546" t="s">
         <v>1648</v>
-      </c>
-      <c r="H546">
-        <v>3</v>
-      </c>
-      <c r="I546" t="s">
-        <v>1649</v>
       </c>
       <c r="J546" t="s">
         <v>99</v>
@@ -32286,7 +32286,7 @@
         <v>21</v>
       </c>
       <c r="L546" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="M546" t="s">
         <v>23</v>
@@ -32300,25 +32300,25 @@
         <v>1500</v>
       </c>
       <c r="C547" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D547" t="s">
         <v>1625</v>
-      </c>
-      <c r="D547" t="s">
-        <v>1626</v>
       </c>
       <c r="E547" t="s">
         <v>52</v>
       </c>
       <c r="F547" t="s">
+        <v>1649</v>
+      </c>
+      <c r="G547" t="s">
         <v>1650</v>
       </c>
-      <c r="G547" t="s">
+      <c r="H547">
+        <v>3</v>
+      </c>
+      <c r="I547" t="s">
         <v>1651</v>
-      </c>
-      <c r="H547">
-        <v>3</v>
-      </c>
-      <c r="I547" t="s">
-        <v>1652</v>
       </c>
       <c r="J547" t="s">
         <v>271</v>
@@ -32341,34 +32341,34 @@
         <v>1500</v>
       </c>
       <c r="C548" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D548" t="s">
         <v>1625</v>
-      </c>
-      <c r="D548" t="s">
-        <v>1626</v>
       </c>
       <c r="E548" t="s">
         <v>52</v>
       </c>
       <c r="F548" t="s">
+        <v>1652</v>
+      </c>
+      <c r="G548" t="s">
         <v>1653</v>
       </c>
-      <c r="G548" t="s">
+      <c r="H548">
+        <v>3</v>
+      </c>
+      <c r="I548" t="s">
         <v>1654</v>
       </c>
-      <c r="H548">
-        <v>3</v>
-      </c>
-      <c r="I548" t="s">
-        <v>1655</v>
-      </c>
       <c r="J548" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="K548" t="s">
         <v>21</v>
       </c>
       <c r="L548" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M548" t="s">
         <v>23</v>
@@ -32382,19 +32382,19 @@
         <v>1500</v>
       </c>
       <c r="C549" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D549" t="s">
         <v>1625</v>
-      </c>
-      <c r="D549" t="s">
-        <v>1626</v>
       </c>
       <c r="E549" t="s">
         <v>52</v>
       </c>
       <c r="F549" t="s">
+        <v>1655</v>
+      </c>
+      <c r="G549" t="s">
         <v>1656</v>
-      </c>
-      <c r="G549" t="s">
-        <v>1657</v>
       </c>
       <c r="H549">
         <v>3</v>
@@ -32409,7 +32409,7 @@
         <v>21</v>
       </c>
       <c r="L549" t="s">
-        <v>1586</v>
+        <v>1516</v>
       </c>
       <c r="M549" t="s">
         <v>23</v>
@@ -32423,34 +32423,34 @@
         <v>1500</v>
       </c>
       <c r="C550" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D550" t="s">
         <v>1625</v>
-      </c>
-      <c r="D550" t="s">
-        <v>1626</v>
       </c>
       <c r="E550" t="s">
         <v>1563</v>
       </c>
       <c r="F550" t="s">
+        <v>1657</v>
+      </c>
+      <c r="G550" t="s">
         <v>1658</v>
-      </c>
-      <c r="G550" t="s">
-        <v>1659</v>
       </c>
       <c r="H550">
         <v>6</v>
       </c>
       <c r="I550" t="s">
+        <v>1659</v>
+      </c>
+      <c r="J550" t="s">
         <v>1660</v>
       </c>
-      <c r="J550" t="s">
-        <v>1661</v>
-      </c>
       <c r="K550" t="s">
         <v>21</v>
       </c>
       <c r="L550" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="M550" t="s">
         <v>23</v>
@@ -32464,25 +32464,25 @@
         <v>1500</v>
       </c>
       <c r="C551" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D551" t="s">
         <v>1625</v>
-      </c>
-      <c r="D551" t="s">
-        <v>1626</v>
       </c>
       <c r="E551" t="s">
         <v>1563</v>
       </c>
       <c r="F551" t="s">
+        <v>1661</v>
+      </c>
+      <c r="G551" t="s">
         <v>1662</v>
       </c>
-      <c r="G551" t="s">
-        <v>1663</v>
-      </c>
       <c r="H551">
         <v>3</v>
       </c>
       <c r="I551" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="J551" t="s">
         <v>148</v>
@@ -32505,25 +32505,25 @@
         <v>1500</v>
       </c>
       <c r="C552" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D552" t="s">
         <v>1625</v>
-      </c>
-      <c r="D552" t="s">
-        <v>1626</v>
       </c>
       <c r="E552" t="s">
         <v>52</v>
       </c>
       <c r="F552" t="s">
+        <v>1663</v>
+      </c>
+      <c r="G552" t="s">
         <v>1664</v>
       </c>
-      <c r="G552" t="s">
+      <c r="H552">
+        <v>3</v>
+      </c>
+      <c r="I552" t="s">
         <v>1665</v>
-      </c>
-      <c r="H552">
-        <v>3</v>
-      </c>
-      <c r="I552" t="s">
-        <v>1666</v>
       </c>
       <c r="J552" t="s">
         <v>271</v>
@@ -32546,25 +32546,25 @@
         <v>1500</v>
       </c>
       <c r="C553" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D553" t="s">
         <v>1625</v>
-      </c>
-      <c r="D553" t="s">
-        <v>1626</v>
       </c>
       <c r="E553" t="s">
         <v>1563</v>
       </c>
       <c r="F553" t="s">
+        <v>1666</v>
+      </c>
+      <c r="G553" t="s">
         <v>1667</v>
       </c>
-      <c r="G553" t="s">
+      <c r="H553">
+        <v>3</v>
+      </c>
+      <c r="I553" t="s">
         <v>1668</v>
-      </c>
-      <c r="H553">
-        <v>3</v>
-      </c>
-      <c r="I553" t="s">
-        <v>1669</v>
       </c>
       <c r="J553" t="s">
         <v>70</v>
@@ -32573,7 +32573,7 @@
         <v>21</v>
       </c>
       <c r="L553" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="M553" t="s">
         <v>23</v>
@@ -32587,19 +32587,19 @@
         <v>1500</v>
       </c>
       <c r="C554" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D554" t="s">
         <v>1625</v>
-      </c>
-      <c r="D554" t="s">
-        <v>1626</v>
       </c>
       <c r="E554" t="s">
         <v>52</v>
       </c>
       <c r="F554" t="s">
+        <v>1669</v>
+      </c>
+      <c r="G554" t="s">
         <v>1670</v>
-      </c>
-      <c r="G554" t="s">
-        <v>1671</v>
       </c>
       <c r="H554">
         <v>3</v>
@@ -32628,19 +32628,19 @@
         <v>1500</v>
       </c>
       <c r="C555" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D555" t="s">
         <v>1625</v>
-      </c>
-      <c r="D555" t="s">
-        <v>1626</v>
       </c>
       <c r="E555" t="s">
         <v>1563</v>
       </c>
       <c r="F555" t="s">
+        <v>1671</v>
+      </c>
+      <c r="G555" t="s">
         <v>1672</v>
-      </c>
-      <c r="G555" t="s">
-        <v>1673</v>
       </c>
       <c r="H555">
         <v>3</v>
@@ -32669,19 +32669,19 @@
         <v>1500</v>
       </c>
       <c r="C556" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D556" t="s">
         <v>1625</v>
-      </c>
-      <c r="D556" t="s">
-        <v>1626</v>
       </c>
       <c r="E556" t="s">
         <v>1563</v>
       </c>
       <c r="F556" t="s">
+        <v>1673</v>
+      </c>
+      <c r="G556" t="s">
         <v>1674</v>
-      </c>
-      <c r="G556" t="s">
-        <v>1675</v>
       </c>
       <c r="H556">
         <v>3</v>
@@ -32710,25 +32710,25 @@
         <v>1500</v>
       </c>
       <c r="C557" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D557" t="s">
         <v>1625</v>
-      </c>
-      <c r="D557" t="s">
-        <v>1626</v>
       </c>
       <c r="E557" t="s">
         <v>1563</v>
       </c>
       <c r="F557" t="s">
+        <v>1675</v>
+      </c>
+      <c r="G557" t="s">
         <v>1676</v>
       </c>
-      <c r="G557" t="s">
-        <v>1677</v>
-      </c>
       <c r="H557">
         <v>3</v>
       </c>
       <c r="I557" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J557" t="s">
         <v>908</v>
@@ -32737,7 +32737,7 @@
         <v>21</v>
       </c>
       <c r="L557" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="M557" t="s">
         <v>23</v>
@@ -32751,25 +32751,25 @@
         <v>1500</v>
       </c>
       <c r="C558" t="s">
+        <v>1624</v>
+      </c>
+      <c r="D558" t="s">
         <v>1625</v>
-      </c>
-      <c r="D558" t="s">
-        <v>1626</v>
       </c>
       <c r="E558" t="s">
         <v>1563</v>
       </c>
       <c r="F558" t="s">
+        <v>1677</v>
+      </c>
+      <c r="G558" t="s">
         <v>1678</v>
       </c>
-      <c r="G558" t="s">
-        <v>1679</v>
-      </c>
       <c r="H558">
         <v>3</v>
       </c>
       <c r="I558" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J558" t="s">
         <v>854</v>
@@ -32792,16 +32792,16 @@
         <v>1500</v>
       </c>
       <c r="C559" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D559" t="s">
         <v>1680</v>
-      </c>
-      <c r="D559" t="s">
-        <v>1681</v>
       </c>
       <c r="E559" t="s">
         <v>52</v>
       </c>
       <c r="F559" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="G559" t="s">
         <v>1540</v>
@@ -32810,7 +32810,7 @@
         <v>0</v>
       </c>
       <c r="I559" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J559" t="s">
         <v>571</v>
@@ -32819,7 +32819,7 @@
         <v>21</v>
       </c>
       <c r="L559" t="s">
-        <v>1586</v>
+        <v>1516</v>
       </c>
       <c r="M559" t="s">
         <v>23</v>
@@ -32833,16 +32833,16 @@
         <v>1500</v>
       </c>
       <c r="C560" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D560" t="s">
         <v>1680</v>
-      </c>
-      <c r="D560" t="s">
-        <v>1681</v>
       </c>
       <c r="E560" t="s">
         <v>52</v>
       </c>
       <c r="F560" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="G560" t="s">
         <v>1549</v>
@@ -32851,7 +32851,7 @@
         <v>3</v>
       </c>
       <c r="I560" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J560" t="s">
         <v>359</v>
@@ -32874,25 +32874,25 @@
         <v>1500</v>
       </c>
       <c r="C561" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D561" t="s">
         <v>1680</v>
-      </c>
-      <c r="D561" t="s">
-        <v>1681</v>
       </c>
       <c r="E561" t="s">
         <v>52</v>
       </c>
       <c r="F561" t="s">
+        <v>1684</v>
+      </c>
+      <c r="G561" t="s">
         <v>1685</v>
       </c>
-      <c r="G561" t="s">
+      <c r="H561">
+        <v>3</v>
+      </c>
+      <c r="I561" t="s">
         <v>1686</v>
-      </c>
-      <c r="H561">
-        <v>3</v>
-      </c>
-      <c r="I561" t="s">
-        <v>1687</v>
       </c>
       <c r="J561" t="s">
         <v>908</v>
@@ -32915,19 +32915,19 @@
         <v>1500</v>
       </c>
       <c r="C562" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D562" t="s">
         <v>1680</v>
-      </c>
-      <c r="D562" t="s">
-        <v>1681</v>
       </c>
       <c r="E562" t="s">
         <v>1563</v>
       </c>
       <c r="F562" t="s">
+        <v>1687</v>
+      </c>
+      <c r="G562" t="s">
         <v>1688</v>
-      </c>
-      <c r="G562" t="s">
-        <v>1689</v>
       </c>
       <c r="H562">
         <v>6</v>
@@ -32936,13 +32936,13 @@
         <v>1519</v>
       </c>
       <c r="J562" t="s">
+        <v>1689</v>
+      </c>
+      <c r="K562" t="s">
+        <v>21</v>
+      </c>
+      <c r="L562" t="s">
         <v>1690</v>
-      </c>
-      <c r="K562" t="s">
-        <v>21</v>
-      </c>
-      <c r="L562" t="s">
-        <v>1506</v>
       </c>
       <c r="M562" t="s">
         <v>23</v>
@@ -32956,10 +32956,10 @@
         <v>1500</v>
       </c>
       <c r="C563" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D563" t="s">
         <v>1680</v>
-      </c>
-      <c r="D563" t="s">
-        <v>1681</v>
       </c>
       <c r="E563" t="s">
         <v>1563</v>
@@ -32983,7 +32983,7 @@
         <v>21</v>
       </c>
       <c r="L563" t="s">
-        <v>1618</v>
+        <v>1617</v>
       </c>
       <c r="M563" t="s">
         <v>23</v>
@@ -32997,10 +32997,10 @@
         <v>1500</v>
       </c>
       <c r="C564" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D564" t="s">
         <v>1680</v>
-      </c>
-      <c r="D564" t="s">
-        <v>1681</v>
       </c>
       <c r="E564" t="s">
         <v>52</v>
@@ -33038,10 +33038,10 @@
         <v>1500</v>
       </c>
       <c r="C565" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D565" t="s">
         <v>1680</v>
-      </c>
-      <c r="D565" t="s">
-        <v>1681</v>
       </c>
       <c r="E565" t="s">
         <v>52</v>
@@ -33056,7 +33056,7 @@
         <v>3</v>
       </c>
       <c r="I565" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J565" t="s">
         <v>908</v>
@@ -33079,10 +33079,10 @@
         <v>1500</v>
       </c>
       <c r="C566" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D566" t="s">
         <v>1680</v>
-      </c>
-      <c r="D566" t="s">
-        <v>1681</v>
       </c>
       <c r="E566" t="s">
         <v>1563</v>
@@ -33120,10 +33120,10 @@
         <v>1500</v>
       </c>
       <c r="C567" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D567" t="s">
         <v>1680</v>
-      </c>
-      <c r="D567" t="s">
-        <v>1681</v>
       </c>
       <c r="E567" t="s">
         <v>52</v>
@@ -33161,10 +33161,10 @@
         <v>1500</v>
       </c>
       <c r="C568" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D568" t="s">
         <v>1680</v>
-      </c>
-      <c r="D568" t="s">
-        <v>1681</v>
       </c>
       <c r="E568" t="s">
         <v>52</v>
@@ -33202,10 +33202,10 @@
         <v>1500</v>
       </c>
       <c r="C569" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D569" t="s">
         <v>1680</v>
-      </c>
-      <c r="D569" t="s">
-        <v>1681</v>
       </c>
       <c r="E569" t="s">
         <v>52</v>
@@ -33243,10 +33243,10 @@
         <v>1500</v>
       </c>
       <c r="C570" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D570" t="s">
         <v>1680</v>
-      </c>
-      <c r="D570" t="s">
-        <v>1681</v>
       </c>
       <c r="E570" t="s">
         <v>52</v>
@@ -33270,7 +33270,7 @@
         <v>21</v>
       </c>
       <c r="L570" t="s">
-        <v>1506</v>
+        <v>1690</v>
       </c>
       <c r="M570" t="s">
         <v>23</v>
@@ -33284,10 +33284,10 @@
         <v>1500</v>
       </c>
       <c r="C571" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D571" t="s">
         <v>1680</v>
-      </c>
-      <c r="D571" t="s">
-        <v>1681</v>
       </c>
       <c r="E571" t="s">
         <v>52</v>
@@ -33311,7 +33311,7 @@
         <v>21</v>
       </c>
       <c r="L571" t="s">
-        <v>1506</v>
+        <v>1690</v>
       </c>
       <c r="M571" t="s">
         <v>23</v>
@@ -33325,10 +33325,10 @@
         <v>1500</v>
       </c>
       <c r="C572" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D572" t="s">
         <v>1680</v>
-      </c>
-      <c r="D572" t="s">
-        <v>1681</v>
       </c>
       <c r="E572" t="s">
         <v>1563</v>
@@ -33352,7 +33352,7 @@
         <v>21</v>
       </c>
       <c r="L572" t="s">
-        <v>1506</v>
+        <v>1690</v>
       </c>
       <c r="M572" t="s">
         <v>23</v>
@@ -33366,10 +33366,10 @@
         <v>1500</v>
       </c>
       <c r="C573" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D573" t="s">
         <v>1680</v>
-      </c>
-      <c r="D573" t="s">
-        <v>1681</v>
       </c>
       <c r="E573" t="s">
         <v>52</v>
@@ -33407,10 +33407,10 @@
         <v>1500</v>
       </c>
       <c r="C574" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D574" t="s">
         <v>1680</v>
-      </c>
-      <c r="D574" t="s">
-        <v>1681</v>
       </c>
       <c r="E574" t="s">
         <v>1563</v>
@@ -33448,10 +33448,10 @@
         <v>1500</v>
       </c>
       <c r="C575" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D575" t="s">
         <v>1680</v>
-      </c>
-      <c r="D575" t="s">
-        <v>1681</v>
       </c>
       <c r="E575" t="s">
         <v>1563</v>
@@ -42773,7 +42773,7 @@
         <v>3</v>
       </c>
       <c r="I802" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J802" t="s">
         <v>355</v>
@@ -42814,7 +42814,7 @@
         <v>3</v>
       </c>
       <c r="I803" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="J803" t="s">
         <v>2415</v>
@@ -43511,7 +43511,7 @@
         <v>3</v>
       </c>
       <c r="I820" t="s">
-        <v>1630</v>
+        <v>1629</v>
       </c>
       <c r="J820" t="s">
         <v>355</v>
@@ -43520,7 +43520,7 @@
         <v>21</v>
       </c>
       <c r="L820" t="s">
-        <v>1631</v>
+        <v>1630</v>
       </c>
       <c r="M820" t="s">
         <v>23</v>
@@ -43552,7 +43552,7 @@
         <v>3</v>
       </c>
       <c r="I821" t="s">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="J821" t="s">
         <v>2415</v>
@@ -45110,7 +45110,7 @@
         <v>2</v>
       </c>
       <c r="I859" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="J859" t="s">
         <v>2638</v>
@@ -47652,7 +47652,7 @@
         <v>2</v>
       </c>
       <c r="I921" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="J921" t="s">
         <v>678</v>

</xml_diff>